<commit_message>
Correct fusion evidence governance findings
</commit_message>
<xml_diff>
--- a/research/fusion-evidence/fusion_source_review_v1.xlsx
+++ b/research/fusion-evidence/fusion_source_review_v1.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START_HERE" sheetId="1" r:id="R5454025bb1c64e6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOURCE_CANDIDATES" sheetId="2" r:id="R66c99387a90a40c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLAIM_SOURCE_MAP" sheetId="3" r:id="Rca6aa8645d9a4844"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROFILE_COVERAGE" sheetId="4" r:id="R2895e18f2ea642e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROMOTION_EXCEPTIONS" sheetId="5" r:id="Rbb114e11e9704217"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REJECTED_DEFERRED" sheetId="6" r:id="R4c62777bc12c4fa9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHANGE_LOG" sheetId="7" r:id="Rdf0f8056159341a0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATA_DICTIONARY" sheetId="8" r:id="R3996931aedba4f22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START_HERE" sheetId="1" r:id="Rc2bc4bb7e8b6479f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOURCE_CANDIDATES" sheetId="2" r:id="R299294285b25407f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CLAIM_SOURCE_MAP" sheetId="3" r:id="R121a4389c3c54c96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROFILE_COVERAGE" sheetId="4" r:id="Rbdfee3e93c1b4883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PROMOTION_EXCEPTIONS" sheetId="5" r:id="R790844c0ef194dad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REJECTED_DEFERRED" sheetId="6" r:id="R3c27d7f35a6145da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHANGE_LOG" sheetId="7" r:id="R3eeb1baf40ab46fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DATA_DICTIONARY" sheetId="8" r:id="R3afb4acd6b2c4127"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -225,8 +225,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceCandidatesTable" displayName="SourceCandidatesTable" ref="A1:AF45" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:AF45"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SourceCandidatesTable" displayName="SourceCandidatesTable" ref="A1:AF47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:AF47"/>
   <x:tableColumns count="32">
     <x:tableColumn id="1" name="pack_source_id"/>
     <x:tableColumn id="2" name="candidate_source_id"/>
@@ -266,8 +266,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClaimSourceMapTable" displayName="ClaimSourceMapTable" ref="A1:W101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:W101"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ClaimSourceMapTable" displayName="ClaimSourceMapTable" ref="A1:W110" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:W110"/>
   <x:tableColumns count="23">
     <x:tableColumn id="1" name="claim_id"/>
     <x:tableColumn id="2" name="profile_id"/>
@@ -362,8 +362,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RejectedDeferredTable" displayName="RejectedDeferredTable" ref="A1:M15" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:M15"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="RejectedDeferredTable" displayName="RejectedDeferredTable" ref="A1:M12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:M12"/>
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="record_id"/>
     <x:tableColumn id="2" name="pack_source_id"/>
@@ -384,8 +384,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ChangeLogTable" displayName="ChangeLogTable" ref="A1:L4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:L4"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ChangeLogTable" displayName="ChangeLogTable" ref="A1:L11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:L11"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="change_id"/>
     <x:tableColumn id="2" name="source_or_claim"/>
@@ -684,8 +684,8 @@
         <x:v>Candidate sources</x:v>
       </x:c>
       <x:c r="B7" s="12" t="n">
-        <x:f>COUNTA(SOURCE_CANDIDATES!B2:B45)</x:f>
-        <x:v>44</x:v>
+        <x:f>COUNTA('SOURCE_CANDIDATES'!B2:B47)</x:f>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="D7" s="15" t="str">
         <x:v>1 · Source verification</x:v>
@@ -708,8 +708,8 @@
         <x:v>Staged recommendations</x:v>
       </x:c>
       <x:c r="B8" s="12" t="n">
-        <x:f>COUNTIF(SOURCE_CANDIDATES!AE2:AE45,"stage")+COUNTIF(SOURCE_CANDIDATES!AE2:AE45,"stage_scope_limited")</x:f>
-        <x:v>40</x:v>
+        <x:f>COUNTIF('SOURCE_CANDIDATES'!AE2:AE47,"stage")+COUNTIF('SOURCE_CANDIDATES'!AE2:AE47,"stage_scope_limited")</x:f>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="D8" s="15" t="str">
         <x:v>2 · Source-register review</x:v>
@@ -732,8 +732,8 @@
         <x:v>Atomic claim rows</x:v>
       </x:c>
       <x:c r="B9" s="12" t="n">
-        <x:f>COUNTA(CLAIM_SOURCE_MAP!A2:A101)</x:f>
-        <x:v>100</x:v>
+        <x:f>COUNTA('CLAIM_SOURCE_MAP'!A2:A110)</x:f>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D9" s="15" t="str">
         <x:v>3 · Fusion domain review</x:v>
@@ -756,7 +756,7 @@
         <x:v>Frozen profile rows</x:v>
       </x:c>
       <x:c r="B10" s="12" t="n">
-        <x:f>COUNTA(PROFILE_COVERAGE!A2:A19)</x:f>
+        <x:f>COUNTA('PROFILE_COVERAGE'!A2:A19)</x:f>
         <x:v>18</x:v>
       </x:c>
       <x:c r="D10" s="15" t="str">
@@ -780,7 +780,7 @@
         <x:v>Claim-level owner exceptions</x:v>
       </x:c>
       <x:c r="B11" s="12" t="n">
-        <x:f>COUNTA(PROMOTION_EXCEPTIONS!A2:A8)</x:f>
+        <x:f>COUNTA('PROMOTION_EXCEPTIONS'!A2:A8)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="D11" s="15" t="str">
@@ -804,6 +804,7 @@
         <x:v>Source corrections</x:v>
       </x:c>
       <x:c r="B12" s="12" t="n">
+        <x:f>COUNTIF('PROMOTION_EXCEPTIONS'!B2:B9,"source_characterization_correction")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="D12" s="15" t="str">
@@ -1331,7 +1332,7 @@
       </x:c>
       <x:c r="AF4" s="31" t="str"/>
     </x:row>
-    <x:row r="5" ht="129.60000610351562" hidden="0" customHeight="1">
+    <x:row r="5" ht="259.20001220703125" hidden="0" customHeight="1">
       <x:c r="A5" s="31" t="str">
         <x:v>S-CN-LAW</x:v>
       </x:c>
@@ -1345,7 +1346,7 @@
         <x:v>Atomic Energy Law of the People's Republic of China</x:v>
       </x:c>
       <x:c r="E5" s="31" t="str">
-        <x:v>National People's Congress (Ministry of Commerce legal database mirror)</x:v>
+        <x:v>National People's Congress / China Atomic Energy Authority republication</x:v>
       </x:c>
       <x:c r="F5" s="31" t="str">
         <x:v>2025-09-12</x:v>
@@ -1378,22 +1379,22 @@
         <x:v>not_applicable</x:v>
       </x:c>
       <x:c r="P5" s="31" t="str">
-        <x:v>https://policy.mofcom.gov.cn/claw/clawContent.shtml?id=103716</x:v>
+        <x:v>https://www.caea.gov.cn/n6760338/n6760344/n10763762/n10763767/c10704020/content.html</x:v>
       </x:c>
       <x:c r="Q5" s="31" t="str">
-        <x:v>https://policy.mofcom.gov.cn/claw/clawContent.shtml?id=103716</x:v>
+        <x:v>https://www.caea.gov.cn/n6760338/n6760344/n10763762/n10763767/c10704020/content.html</x:v>
       </x:c>
       <x:c r="R5" s="31" t="str">
         <x:v>missing</x:v>
       </x:c>
       <x:c r="S5" s="31" t="str">
-        <x:v>Article number and dates checked in the Chinese legal text; legal interpretation requires a qualified reviewer.</x:v>
+        <x:v>Final-law locators checked against the official Chinese full text: Articles 14 and 39. Earlier draft numbering must not be used as the final-law locator; legal interpretation requires a qualified reviewer.</x:v>
       </x:c>
       <x:c r="T5" s="31" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="U5" s="31" t="str">
-        <x:v>programme announcement</x:v>
+        <x:v>observed legal/regulatory status</x:v>
       </x:c>
       <x:c r="V5" s="31" t="str">
         <x:v>China</x:v>
@@ -1411,13 +1412,13 @@
         <x:v>S2;S3;S4;S5</x:v>
       </x:c>
       <x:c r="AA5" s="31" t="str">
-        <x:v>The law includes controlled thermonuclear fusion within the national atomic-energy legal framework.</x:v>
+        <x:v>The final law encourages and supports controlled-thermonuclear-fusion R&amp;D in Article 14 and establishes a fusion-suited regulatory system with graded/classified management in Article 39.</x:v>
       </x:c>
       <x:c r="AB5" s="31" t="str">
-        <x:v>Effective 2026-01-15; promulgation and effective dates in header. Controlled thermonuclear fusion provision: Article 37.</x:v>
+        <x:v>Adopted 2025-09-12; page heading. Effective 2026-01-15; Article 62. Fusion R&amp;D support: Article 14. Fusion-specific supervision and graded/classified management of fusion fuels and devices/facilities: Article 39.</x:v>
       </x:c>
       <x:c r="AC5" s="31" t="str">
-        <x:v>A statute establishes authority and duties; it is not a completed fusion licensing case or evidence of review duration.</x:v>
+        <x:v>An enacted law establishes legal status and authority; it is not a completed fusion licensing case or evidence of review duration. Earlier draft numbering differed, and final Article 37 concerns disused radioactive-source recovery/disposal.</x:v>
       </x:c>
       <x:c r="AD5" s="31" t="str">
         <x:v>verified_official_primary</x:v>
@@ -3155,7 +3156,7 @@
       </x:c>
       <x:c r="AF23" s="31" t="str"/>
     </x:row>
-    <x:row r="24" ht="108" hidden="0" customHeight="1">
+    <x:row r="24" ht="356.3999938964844" hidden="0" customHeight="1">
       <x:c r="A24" s="31" t="str">
         <x:v>unassigned_pack_table</x:v>
       </x:c>
@@ -3163,16 +3164,16 @@
         <x:v>fusion-src-023</x:v>
       </x:c>
       <x:c r="C24" s="31" t="str">
-        <x:v>HEAT-ML research highlight</x:v>
+        <x:v>Finding the shadows in a fusion system faster with AI</x:v>
       </x:c>
       <x:c r="D24" s="31" t="str">
-        <x:v>HEAT-ML research highlight</x:v>
+        <x:v>Finding the shadows in a fusion system faster with AI</x:v>
       </x:c>
       <x:c r="E24" s="31" t="str">
-        <x:v>Princeton Plasma Physics Laboratory</x:v>
+        <x:v>Corona Rivera et al.; Princeton Plasma Physics Laboratory / Fusion Engineering and Design</x:v>
       </x:c>
       <x:c r="F24" s="31" t="str">
-        <x:v>missing</x:v>
+        <x:v>2025-08-13</x:v>
       </x:c>
       <x:c r="G24" s="31" t="str">
         <x:v>2026-08-31</x:v>
@@ -3190,19 +3191,19 @@
         <x:v>official_research_highlight</x:v>
       </x:c>
       <x:c r="L24" s="31" t="str">
-        <x:v>expert_commentary</x:v>
+        <x:v>peer_reviewed_paper</x:v>
       </x:c>
       <x:c r="M24" s="31" t="str">
-        <x:v>official_research_institute</x:v>
+        <x:v>research_authors</x:v>
       </x:c>
       <x:c r="N24" s="31" t="str">
-        <x:v>official_program_claim</x:v>
+        <x:v>not_official_claim</x:v>
       </x:c>
       <x:c r="O24" s="31" t="str">
-        <x:v>unknown</x:v>
+        <x:v>independently_validated</x:v>
       </x:c>
       <x:c r="P24" s="31" t="str">
-        <x:v>https://www.pppl.gov/news/2026</x:v>
+        <x:v>https://www.pppl.gov/news/2025/finding-shadows-fusion-system-faster-ai</x:v>
       </x:c>
       <x:c r="Q24" s="31" t="str">
         <x:v>missing</x:v>
@@ -3214,7 +3215,7 @@
         <x:v>not_applicable</x:v>
       </x:c>
       <x:c r="T24" s="31" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="U24" s="31" t="str">
         <x:v>proof of concept</x:v>
@@ -3226,31 +3227,31 @@
         <x:v>tokamak_research_to_pilot_plant_demonstration</x:v>
       </x:c>
       <x:c r="X24" s="31" t="str">
-        <x:v>simulation;plasma_facing_components</x:v>
+        <x:v>simulation</x:v>
       </x:c>
       <x:c r="Y24" s="31" t="str">
-        <x:v>sp-0015;sp-0023</x:v>
+        <x:v>sp-0015</x:v>
       </x:c>
       <x:c r="Z24" s="31" t="str">
         <x:v>S1;S2;S3</x:v>
       </x:c>
       <x:c r="AA24" s="31" t="str">
-        <x:v>The pack describes a surrogate for magnetic-shadow calculations relevant to plasma-facing components.</x:v>
+        <x:v>HEAT-ML is a scoped surrogate for SPARC magnetic-shadow calculations, reducing one geometry-specific calculation from around 30 minutes to a few milliseconds.</x:v>
       </x:c>
       <x:c r="AB24" s="31" t="str">
-        <x:v>missing; the pack did not supply a DOI and the bounded verification pass did not recover a stable article URL.</x:v>
+        <x:v>Around 30 minutes for one conventional HEAT simulation and longer for complex geometry; PPPL paragraphs 101-102. A few milliseconds with HEAT-ML and approximately 1,000 SPARC HEAT simulations in the training database; paragraph 102. Peer-reviewed DOI: https://doi.org/10.1016/j.fusengdes.2025.115010.</x:v>
       </x:c>
       <x:c r="AC24" s="31" t="str">
-        <x:v>Publisher page/DOI and exact paper title were not stably verified.</x:v>
+        <x:v>The present method covers 15 tiles in a small part of SPARC's exhaust geometry and is tied to that design; it is not plant-level schedule acceleration, materials qualification, or a generic plasma-facing-component result.</x:v>
       </x:c>
       <x:c r="AD24" s="31" t="str">
-        <x:v>unverified_locator</x:v>
+        <x:v>verified_peer_reviewed</x:v>
       </x:c>
       <x:c r="AE24" s="31" t="str">
-        <x:v>defer</x:v>
+        <x:v>stage_scope_limited</x:v>
       </x:c>
       <x:c r="AF24" s="31" t="str">
-        <x:v>No promotion until the original PPPL article and Fusion Engineering and Design DOI resolve.</x:v>
+        <x:v>Exact PPPL publisher locator verified; linked paper: Fusion Engineering and Design 217 (2025) 115010, DOI 10.1016/j.fusengdes.2025.115010.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="172.8000030517578" hidden="0" customHeight="1">
@@ -3829,7 +3830,7 @@
       </x:c>
       <x:c r="AF30" s="31" t="str"/>
     </x:row>
-    <x:row r="31" ht="108" hidden="0" customHeight="1">
+    <x:row r="31" ht="183.60000610351562" hidden="0" customHeight="1">
       <x:c r="A31" s="31" t="str">
         <x:v>S-US-NSTXU</x:v>
       </x:c>
@@ -3837,16 +3838,16 @@
         <x:v>fusion-src-030</x:v>
       </x:c>
       <x:c r="C31" s="31" t="str">
-        <x:v>Delivery of magnet bundle signals new age of fusion research</x:v>
+        <x:v>National Spherical Torus Experiment-Upgrade (NSTX-U)</x:v>
       </x:c>
       <x:c r="D31" s="31" t="str">
-        <x:v>Delivery of magnet bundle signals new age of fusion research</x:v>
+        <x:v>National Spherical Torus Experiment-Upgrade (NSTX-U)</x:v>
       </x:c>
       <x:c r="E31" s="31" t="str">
         <x:v>Princeton Plasma Physics Laboratory</x:v>
       </x:c>
       <x:c r="F31" s="31" t="str">
-        <x:v>2026-06-08</x:v>
+        <x:v>missing</x:v>
       </x:c>
       <x:c r="G31" s="31" t="str">
         <x:v>2026-08-31</x:v>
@@ -3861,7 +3862,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="K31" s="31" t="str">
-        <x:v>official_facility_release</x:v>
+        <x:v>official_project_status_page</x:v>
       </x:c>
       <x:c r="L31" s="31" t="str">
         <x:v>administrative_data</x:v>
@@ -3870,13 +3871,13 @@
         <x:v>official_research_institute</x:v>
       </x:c>
       <x:c r="N31" s="31" t="str">
-        <x:v>official_target</x:v>
+        <x:v>official_observed_statistic</x:v>
       </x:c>
       <x:c r="O31" s="31" t="str">
         <x:v>not_applicable</x:v>
       </x:c>
       <x:c r="P31" s="31" t="str">
-        <x:v>https://www.pppl.gov/news/2026/delivery-magnet-bundle-signals-new-age-fusion-research</x:v>
+        <x:v>https://www.pppl.gov/nstx-u</x:v>
       </x:c>
       <x:c r="Q31" s="31" t="str">
         <x:v>missing</x:v>
@@ -3891,7 +3892,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="U31" s="31" t="str">
-        <x:v>official target</x:v>
+        <x:v>observed facility milestone</x:v>
       </x:c>
       <x:c r="V31" s="31" t="str">
         <x:v>United States</x:v>
@@ -3900,22 +3901,22 @@
         <x:v>tokamak_research_to_pilot_plant_demonstration</x:v>
       </x:c>
       <x:c r="X31" s="31" t="str">
-        <x:v>magnets;component_fabrication;construction;commissioning</x:v>
+        <x:v>construction;commissioning</x:v>
       </x:c>
       <x:c r="Y31" s="31" t="str">
-        <x:v>sp-0021;sp-0026;sp-0027;sp-0028</x:v>
+        <x:v>sp-0027;sp-0028</x:v>
       </x:c>
       <x:c r="Z31" s="31" t="str">
-        <x:v>S2;S3;S4;S5</x:v>
+        <x:v>S2;S3;S4</x:v>
       </x:c>
       <x:c r="AA31" s="31" t="str">
-        <x:v>PPPL reports delivery of the central magnet bundle and now expects experiments in 2027.</x:v>
+        <x:v>PPPL's living project page states that the NSTX-U Recovery Project is 93% complete.</x:v>
       </x:c>
       <x:c r="AB31" s="31" t="str">
-        <x:v>2027 experiment target; article lead/body.</x:v>
+        <x:v>93% Recovery Project completion status; section 'Recovery Project', checked 2026-08-31.</x:v>
       </x:c>
       <x:c r="AC31" s="31" t="str">
-        <x:v>Target, not completed recommissioning; the pack's 93% figure was not located on this page and is not promoted.</x:v>
+        <x:v>Living-page project status, not a fixed historical statistic, completed recommissioning, or an experimental outcome.</x:v>
       </x:c>
       <x:c r="AD31" s="31" t="str">
         <x:v>verified_official_primary</x:v>
@@ -3923,7 +3924,9 @@
       <x:c r="AE31" s="31" t="str">
         <x:v>stage_scope_limited</x:v>
       </x:c>
-      <x:c r="AF31" s="31" t="str"/>
+      <x:c r="AF31" s="31" t="str">
+        <x:v>Freshness trigger: recheck before promotion and whenever PPPL changes the Recovery Project timeline/status or announces recommissioning or experiments.</x:v>
+      </x:c>
     </x:row>
     <x:row r="32" ht="97.19999694824219" hidden="0" customHeight="1">
       <x:c r="A32" s="31" t="str">
@@ -4505,7 +4508,7 @@
       </x:c>
       <x:c r="AF37" s="31" t="str"/>
     </x:row>
-    <x:row r="38" ht="162" hidden="0" customHeight="1">
+    <x:row r="38" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A38" s="31" t="str">
         <x:v>S-ITER-2026</x:v>
       </x:c>
@@ -4513,16 +4516,16 @@
         <x:v>fusion-src-037</x:v>
       </x:c>
       <x:c r="C38" s="31" t="str">
-        <x:v>ITER Machine Assembly Overview</x:v>
+        <x:v>Millions of data points, one successful lift</x:v>
       </x:c>
       <x:c r="D38" s="31" t="str">
-        <x:v>ITER Machine Assembly Overview</x:v>
+        <x:v>Millions of data points, one successful lift</x:v>
       </x:c>
       <x:c r="E38" s="31" t="str">
         <x:v>ITER Organization</x:v>
       </x:c>
       <x:c r="F38" s="31" t="str">
-        <x:v>missing</x:v>
+        <x:v>2026-07-29</x:v>
       </x:c>
       <x:c r="G38" s="31" t="str">
         <x:v>2026-08-31</x:v>
@@ -4537,7 +4540,7 @@
         <x:v>en</x:v>
       </x:c>
       <x:c r="K38" s="31" t="str">
-        <x:v>official_program_page</x:v>
+        <x:v>official_facility_release</x:v>
       </x:c>
       <x:c r="L38" s="31" t="str">
         <x:v>administrative_data</x:v>
@@ -4546,13 +4549,13 @@
         <x:v>international_program</x:v>
       </x:c>
       <x:c r="N38" s="31" t="str">
-        <x:v>official_program_claim</x:v>
+        <x:v>official_observed_statistic</x:v>
       </x:c>
       <x:c r="O38" s="31" t="str">
         <x:v>not_applicable</x:v>
       </x:c>
       <x:c r="P38" s="31" t="str">
-        <x:v>https://www.iter.org/project/assembly-overview</x:v>
+        <x:v>https://www.iter.org/node/20687/millions-data-points-one-successful-lift</x:v>
       </x:c>
       <x:c r="Q38" s="31" t="str">
         <x:v>missing</x:v>
@@ -4576,28 +4579,28 @@
         <x:v>tokamak_research_to_pilot_plant_demonstration</x:v>
       </x:c>
       <x:c r="X38" s="31" t="str">
-        <x:v>component_fabrication;construction;commissioning</x:v>
+        <x:v>construction</x:v>
       </x:c>
       <x:c r="Y38" s="31" t="str">
-        <x:v>sp-0026;sp-0027;sp-0028</x:v>
+        <x:v>sp-0027</x:v>
       </x:c>
       <x:c r="Z38" s="31" t="str">
         <x:v>S2;S3;S4</x:v>
       </x:c>
       <x:c r="AA38" s="31" t="str">
-        <x:v>The current page documents the assembly/commissioning topology but does not substantiate the pack's 'sixth of nine sectors' July-2026 numerical claim.</x:v>
+        <x:v>ITER reports that its sixth of nine tokamak sector modules landed in the pit on 28 July 2026, putting two-thirds of the plasma chamber in place.</x:v>
       </x:c>
       <x:c r="AB38" s="31" t="str">
-        <x:v>missing for sixth-of-nine claim; no precise locator recovered on the stable page.</x:v>
+        <x:v>Lift ran 27-28 July 2026; article paragraphs 162-167. Sixth of nine modules and two-thirds of chamber in place; paragraphs 162 and 167. The official project milestone page https://www.iter.org/project/road-iter also records the sixth-module milestone.</x:v>
       </x:c>
       <x:c r="AC38" s="31" t="str">
-        <x:v>Use for phase definitions only; defer the July-2026 sector-count claim pending the exact original news page.</x:v>
+        <x:v>Observed construction/facility milestone only; not an AI result, integrated chamber completion, commissioning, or plant completion.</x:v>
       </x:c>
       <x:c r="AD38" s="31" t="str">
-        <x:v>partially_verified_scope_only</x:v>
+        <x:v>verified_official_primary</x:v>
       </x:c>
       <x:c r="AE38" s="31" t="str">
-        <x:v>defer</x:v>
+        <x:v>stage_scope_limited</x:v>
       </x:c>
       <x:c r="AF38" s="31" t="str"/>
     </x:row>
@@ -4697,7 +4700,7 @@
       </x:c>
       <x:c r="AF39" s="31" t="str"/>
     </x:row>
-    <x:row r="40" ht="140.39999389648438" hidden="0" customHeight="1">
+    <x:row r="40" ht="151.1999969482422" hidden="0" customHeight="1">
       <x:c r="A40" s="31" t="str">
         <x:v>S-US-NRC</x:v>
       </x:c>
@@ -4759,7 +4762,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="U40" s="31" t="str">
-        <x:v>programme announcement</x:v>
+        <x:v>observed legal/regulatory status</x:v>
       </x:c>
       <x:c r="V40" s="31" t="str">
         <x:v>United States</x:v>
@@ -4777,13 +4780,13 @@
         <x:v>S2;S3;S4;S5</x:v>
       </x:c>
       <x:c r="AA40" s="31" t="str">
-        <x:v>The NRC proposed a Part 30-based, technology-neutral licensing framework for fusion machines.</x:v>
+        <x:v>The NRC published a proposed Part 30-based, technology-neutral licensing framework for fusion machines.</x:v>
       </x:c>
       <x:c r="AB40" s="31" t="str">
-        <x:v>91 FR 9476; Federal Register citation and document header. 90-day comment period ending 2026-05-27; Dates section.</x:v>
+        <x:v>91 FR 9476; Federal Register citation and document header. 90-day rulemaking comment period ending 2026-05-27; Dates section.</x:v>
       </x:c>
       <x:c r="AC40" s="31" t="str">
-        <x:v>Proposed rule and draft guidance, not a final rule or an observed plant licence review.</x:v>
+        <x:v>Proposed rule and draft guidance, not a final rule, observed plant-licence review, or licence-review-duration dataset.</x:v>
       </x:c>
       <x:c r="AD40" s="31" t="str">
         <x:v>verified_official_primary</x:v>
@@ -4793,7 +4796,7 @@
       </x:c>
       <x:c r="AF40" s="31" t="str"/>
     </x:row>
-    <x:row r="41" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="41" ht="129.60000610351562" hidden="0" customHeight="1">
       <x:c r="A41" s="31" t="str">
         <x:v>S-US-NRC</x:v>
       </x:c>
@@ -4855,7 +4858,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="U41" s="31" t="str">
-        <x:v>programme announcement</x:v>
+        <x:v>observed legal/regulatory status</x:v>
       </x:c>
       <x:c r="V41" s="31" t="str">
         <x:v>United States</x:v>
@@ -4879,7 +4882,7 @@
         <x:v>Page Last Reviewed/Updated 2026-08-27; footer. Proposed-rule milestone 2026-02-26; table.</x:v>
       </x:c>
       <x:c r="AC41" s="31" t="str">
-        <x:v>Regulatory status, not evidence of licence throughput or a completed plant application.</x:v>
+        <x:v>Current regulator status, not evidence of licence throughput, a completed plant application, or licence-review duration.</x:v>
       </x:c>
       <x:c r="AD41" s="31" t="str">
         <x:v>verified_official_primary</x:v>
@@ -5277,10 +5280,202 @@
       </x:c>
       <x:c r="AF45" s="31" t="str"/>
     </x:row>
+    <x:row r="46" ht="270" hidden="0" customHeight="1">
+      <x:c r="A46" s="31" t="str">
+        <x:v>targeted_ifmif_dones</x:v>
+      </x:c>
+      <x:c r="B46" s="31" t="str">
+        <x:v>fusion-src-045</x:v>
+      </x:c>
+      <x:c r="C46" s="31" t="str">
+        <x:v>The IFMIF-DONES Irradiation Modules</x:v>
+      </x:c>
+      <x:c r="D46" s="31" t="str">
+        <x:v>The IFMIF-DONES Irradiation Modules</x:v>
+      </x:c>
+      <x:c r="E46" s="31" t="str">
+        <x:v>Arbeiter et al.; Nuclear Fusion</x:v>
+      </x:c>
+      <x:c r="F46" s="31" t="str">
+        <x:v>2025-09-30</x:v>
+      </x:c>
+      <x:c r="G46" s="31" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="H46" s="31" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="I46" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="J46" s="31" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="K46" s="31" t="str">
+        <x:v>peer_reviewed_paper</x:v>
+      </x:c>
+      <x:c r="L46" s="31" t="str">
+        <x:v>peer_reviewed_paper</x:v>
+      </x:c>
+      <x:c r="M46" s="31" t="str">
+        <x:v>research_authors</x:v>
+      </x:c>
+      <x:c r="N46" s="31" t="str">
+        <x:v>not_official_claim</x:v>
+      </x:c>
+      <x:c r="O46" s="31" t="str">
+        <x:v>independently_validated</x:v>
+      </x:c>
+      <x:c r="P46" s="31" t="str">
+        <x:v>https://doi.org/10.1088/1741-4326/add172</x:v>
+      </x:c>
+      <x:c r="Q46" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="R46" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="S46" s="31" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="T46" s="31" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="U46" s="31" t="str">
+        <x:v>model or scenario estimate</x:v>
+      </x:c>
+      <x:c r="V46" s="31" t="str">
+        <x:v>European Union;Spain</x:v>
+      </x:c>
+      <x:c r="W46" s="31" t="str">
+        <x:v>tokamak_research_to_pilot_plant_demonstration</x:v>
+      </x:c>
+      <x:c r="X46" s="31" t="str">
+        <x:v>materials_qualification</x:v>
+      </x:c>
+      <x:c r="Y46" s="31" t="str">
+        <x:v>sp-0020</x:v>
+      </x:c>
+      <x:c r="Z46" s="31" t="str">
+        <x:v>S2;S3;S4</x:v>
+      </x:c>
+      <x:c r="AA46" s="31" t="str">
+        <x:v>The peer-reviewed design describes IFMIF-DONES irradiation modules intended to produce future fusion-like materials data, including the HFTM and post-irradiation examination chain.</x:v>
+      </x:c>
+      <x:c r="AB46" s="31" t="str">
+        <x:v>HFTM expects up to 50 dpa in 3 years in a limited volume at 250-550 °C; HFTM section. Post-irradiation examination steps; TRTM and conclusions sections. DOI 10.1088/1741-4326/add172.</x:v>
+      </x:c>
+      <x:c r="AC46" s="31" t="str">
+        <x:v>IFMIF-DONES and its modules are under design/development; no completed or accepted qualification dataset exists. Spectrum/transmutation matching is material-dependent: Eurofer is tailored, while tungsten/copper conditions are not perfectly matched.</x:v>
+      </x:c>
+      <x:c r="AD46" s="31" t="str">
+        <x:v>verified_peer_reviewed</x:v>
+      </x:c>
+      <x:c r="AE46" s="31" t="str">
+        <x:v>stage_scope_limited</x:v>
+      </x:c>
+      <x:c r="AF46" s="31" t="str"/>
+    </x:row>
+    <x:row r="47" ht="248.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A47" s="31" t="str">
+        <x:v>targeted_ifmif_dones</x:v>
+      </x:c>
+      <x:c r="B47" s="31" t="str">
+        <x:v>fusion-src-046</x:v>
+      </x:c>
+      <x:c r="C47" s="31" t="str">
+        <x:v>IFMIF-DONES: Experimental strategy for fusion materials qualification</x:v>
+      </x:c>
+      <x:c r="D47" s="31" t="str">
+        <x:v>IFMIF-DONES: Experimental strategy for fusion materials qualification</x:v>
+      </x:c>
+      <x:c r="E47" s="31" t="str">
+        <x:v>Angel Ibarra / IFMIF-DONES; International Atomic Energy Agency technical meeting</x:v>
+      </x:c>
+      <x:c r="F47" s="31" t="str">
+        <x:v>2025-09-04</x:v>
+      </x:c>
+      <x:c r="G47" s="31" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="H47" s="31" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="I47" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="J47" s="31" t="str">
+        <x:v>en</x:v>
+      </x:c>
+      <x:c r="K47" s="31" t="str">
+        <x:v>official_meeting_contribution</x:v>
+      </x:c>
+      <x:c r="L47" s="31" t="str">
+        <x:v>government_strategy</x:v>
+      </x:c>
+      <x:c r="M47" s="31" t="str">
+        <x:v>international_program</x:v>
+      </x:c>
+      <x:c r="N47" s="31" t="str">
+        <x:v>official_target</x:v>
+      </x:c>
+      <x:c r="O47" s="31" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="P47" s="31" t="str">
+        <x:v>https://conferences.iaea.org/event/406/contributions/37622/</x:v>
+      </x:c>
+      <x:c r="Q47" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="R47" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="S47" s="31" t="str">
+        <x:v>not_applicable</x:v>
+      </x:c>
+      <x:c r="T47" s="31" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="U47" s="31" t="str">
+        <x:v>official target</x:v>
+      </x:c>
+      <x:c r="V47" s="31" t="str">
+        <x:v>European Union;Spain</x:v>
+      </x:c>
+      <x:c r="W47" s="31" t="str">
+        <x:v>tokamak_research_to_pilot_plant_demonstration</x:v>
+      </x:c>
+      <x:c r="X47" s="31" t="str">
+        <x:v>materials_qualification</x:v>
+      </x:c>
+      <x:c r="Y47" s="31" t="str">
+        <x:v>sp-0020</x:v>
+      </x:c>
+      <x:c r="Z47" s="31" t="str">
+        <x:v>S2;S3;S4</x:v>
+      </x:c>
+      <x:c r="AA47" s="31" t="str">
+        <x:v>The official technical contribution describes the planned accelerator-driven fusion-like neutron spectrum, HFTM irradiation campaigns, and the role of the resulting data in materials qualification.</x:v>
+      </x:c>
+      <x:c r="AB47" s="31" t="str">
+        <x:v>Up to 20-30 dpa over 2.5 full-power years in 300 cm3 and 50 dpa in 3 full-power years in 100 cm3; Description paragraphs 1-2. Expected operational date 2034; Description paragraph 1.</x:v>
+      </x:c>
+      <x:c r="AC47" s="31" t="str">
+        <x:v>The facility is under construction and the values are programme design targets, not observed irradiation campaigns or a completed accepted qualification dataset. Post-irradiation examination remains part of the qualification chain.</x:v>
+      </x:c>
+      <x:c r="AD47" s="31" t="str">
+        <x:v>verified_official_primary</x:v>
+      </x:c>
+      <x:c r="AE47" s="31" t="str">
+        <x:v>stage_scope_limited</x:v>
+      </x:c>
+      <x:c r="AF47" s="31" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4bb3621a63da4ba6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R951c72c7c07d47b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5766,7 +5961,7 @@
         <x:v>S-CN-HL3-AI;S-AI-TCV;unassigned_pack_table;S-US-STELLAR</x:v>
       </x:c>
       <x:c r="I7" s="31" t="str">
-        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-024</x:v>
+        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-023;fusion-src-024</x:v>
       </x:c>
       <x:c r="J7" s="31" t="str">
         <x:v>supports</x:v>
@@ -5837,7 +6032,7 @@
         <x:v>S-CN-HL3-AI;S-AI-TCV;unassigned_pack_table;S-US-STELLAR</x:v>
       </x:c>
       <x:c r="I8" s="31" t="str">
-        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-024</x:v>
+        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-023;fusion-src-024</x:v>
       </x:c>
       <x:c r="J8" s="31" t="str">
         <x:v>supports_with_limits</x:v>
@@ -5908,7 +6103,7 @@
         <x:v>S-CN-HL3-AI;S-AI-TCV;unassigned_pack_table;S-US-STELLAR</x:v>
       </x:c>
       <x:c r="I9" s="31" t="str">
-        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-024</x:v>
+        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-023;fusion-src-024</x:v>
       </x:c>
       <x:c r="J9" s="31" t="str">
         <x:v>supports_with_limits</x:v>
@@ -5979,7 +6174,7 @@
         <x:v>S-CN-HL3-AI;S-AI-TCV;unassigned_pack_table;S-US-STELLAR</x:v>
       </x:c>
       <x:c r="I10" s="31" t="str">
-        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-024</x:v>
+        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-023;fusion-src-024</x:v>
       </x:c>
       <x:c r="J10" s="31" t="str">
         <x:v>complicates</x:v>
@@ -7538,10 +7733,10 @@
         <x:v>inference</x:v>
       </x:c>
       <x:c r="H32" s="31" t="str">
-        <x:v>S-CN-ROADMAP;S-US-MPEX;S-US-MPEX-AI;S-US-DOE-ROAD;S-US-DCP;S-ITER-TRITIUM</x:v>
+        <x:v>targeted_ifmif_dones;S-CN-ROADMAP;S-US-MPEX;S-US-MPEX-AI;S-US-DOE-ROAD;S-US-DCP;S-ITER-TRITIUM</x:v>
       </x:c>
       <x:c r="I32" s="31" t="str">
-        <x:v>fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
+        <x:v>fusion-src-046;fusion-src-045;fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
       </x:c>
       <x:c r="J32" s="31" t="str">
         <x:v>supports_with_limits</x:v>
@@ -7586,7 +7781,7 @@
         <x:v>Coverage statement only; this row does not select or recode an S value.</x:v>
       </x:c>
     </x:row>
-    <x:row r="33" ht="162" hidden="0" customHeight="1">
+    <x:row r="33" ht="226.8000030517578" hidden="0" customHeight="1">
       <x:c r="A33" s="31" t="str">
         <x:v>fusion-clm-032</x:v>
       </x:c>
@@ -7600,34 +7795,34 @@
         <x:v>S2</x:v>
       </x:c>
       <x:c r="E33" s="31" t="str">
-        <x:v>The verified source set complicates any simple claim about feedback speed for Materials qualification; physical scope and lifecycle distinctions remain load-bearing.</x:v>
+        <x:v>IFMIF-DONES design and programme-target sources directly establish a planned multi-year irradiation-and-post-irradiation-examination feedback chain for materials qualification; they do not report a completed dataset.</x:v>
       </x:c>
       <x:c r="F33" s="31" t="str">
-        <x:v>inference</x:v>
+        <x:v>official target</x:v>
       </x:c>
       <x:c r="G33" s="31" t="str">
-        <x:v>inference</x:v>
+        <x:v>official target</x:v>
       </x:c>
       <x:c r="H33" s="31" t="str">
-        <x:v>S-CN-ROADMAP;S-US-MPEX;S-US-MPEX-AI;S-US-DOE-ROAD;S-US-DCP;S-ITER-TRITIUM</x:v>
+        <x:v>targeted_ifmif_dones;S-CN-ROADMAP;S-US-MPEX;S-US-MPEX-AI;S-US-DOE-ROAD;S-US-DCP;S-ITER-TRITIUM</x:v>
       </x:c>
       <x:c r="I33" s="31" t="str">
-        <x:v>fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
+        <x:v>fusion-src-046;fusion-src-045;fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
       </x:c>
       <x:c r="J33" s="31" t="str">
-        <x:v>complicates</x:v>
+        <x:v>supports</x:v>
       </x:c>
       <x:c r="K33" s="31" t="str">
-        <x:v>indirect</x:v>
+        <x:v>direct</x:v>
       </x:c>
       <x:c r="L33" s="31" t="str">
-        <x:v>partial</x:v>
+        <x:v>exact_stage</x:v>
       </x:c>
       <x:c r="M33" s="31" t="str">
         <x:v>frozen_tokamak_pathway</x:v>
       </x:c>
       <x:c r="N33" s="31" t="str">
-        <x:v>partial</x:v>
+        <x:v>designed_under_development_not_completed</x:v>
       </x:c>
       <x:c r="O33" s="31" t="str">
         <x:v>missing</x:v>
@@ -7657,7 +7852,7 @@
         <x:v>Coverage statement only; this row does not select or recode an S value.</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="183.60000610351562" hidden="0" customHeight="1">
+    <x:row r="34" ht="205.1999969482422" hidden="0" customHeight="1">
       <x:c r="A34" s="31" t="str">
         <x:v>fusion-clm-033</x:v>
       </x:c>
@@ -7671,7 +7866,7 @@
         <x:v>S3</x:v>
       </x:c>
       <x:c r="E34" s="31" t="str">
-        <x:v>The verified source set complicates any simple claim about experiment affordability and throughput for Materials qualification; physical scope and lifecycle distinctions remain load-bearing.</x:v>
+        <x:v>IFMIF-DONES planned irradiation volumes and modular campaigns inform qualification throughput only indirectly; they do not establish observed affordability, completed throughput, or acceptance.</x:v>
       </x:c>
       <x:c r="F34" s="31" t="str">
         <x:v>inference</x:v>
@@ -7680,13 +7875,13 @@
         <x:v>inference</x:v>
       </x:c>
       <x:c r="H34" s="31" t="str">
-        <x:v>S-CN-ROADMAP;S-US-MPEX;S-US-MPEX-AI;S-US-DOE-ROAD;S-US-DCP;S-ITER-TRITIUM</x:v>
+        <x:v>targeted_ifmif_dones;S-CN-ROADMAP;S-US-MPEX;S-US-MPEX-AI;S-US-DOE-ROAD;S-US-DCP;S-ITER-TRITIUM</x:v>
       </x:c>
       <x:c r="I34" s="31" t="str">
-        <x:v>fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
+        <x:v>fusion-src-046;fusion-src-045;fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
       </x:c>
       <x:c r="J34" s="31" t="str">
-        <x:v>complicates</x:v>
+        <x:v>supports_with_limits</x:v>
       </x:c>
       <x:c r="K34" s="31" t="str">
         <x:v>indirect</x:v>
@@ -7728,7 +7923,7 @@
         <x:v>Coverage statement only; this row does not select or recode an S value.</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="162" hidden="0" customHeight="1">
+    <x:row r="35" ht="237.60000610351562" hidden="0" customHeight="1">
       <x:c r="A35" s="31" t="str">
         <x:v>fusion-clm-034</x:v>
       </x:c>
@@ -7742,19 +7937,19 @@
         <x:v>S4</x:v>
       </x:c>
       <x:c r="E35" s="31" t="str">
-        <x:v>The verified source set directly informs physical flexibility or elapsed-time floors for Materials qualification within the frozen research-to-pilot pathway.</x:v>
+        <x:v>IFMIF-DONES design and programme-target sources directly support a substantial physical materials-qualification time floor: roughly 2.5-3 full-power years of irradiation before the remaining examination and acceptance chain.</x:v>
       </x:c>
       <x:c r="F35" s="31" t="str">
-        <x:v>commentary</x:v>
+        <x:v>official target</x:v>
       </x:c>
       <x:c r="G35" s="31" t="str">
-        <x:v>commentary</x:v>
+        <x:v>official target</x:v>
       </x:c>
       <x:c r="H35" s="31" t="str">
-        <x:v>S-CN-ROADMAP;S-US-MPEX;S-US-MPEX-AI;S-US-DOE-ROAD;S-US-DCP;S-ITER-TRITIUM</x:v>
+        <x:v>targeted_ifmif_dones;S-CN-ROADMAP;S-US-MPEX;S-US-MPEX-AI;S-US-DOE-ROAD;S-US-DCP;S-ITER-TRITIUM</x:v>
       </x:c>
       <x:c r="I35" s="31" t="str">
-        <x:v>fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
+        <x:v>fusion-src-046;fusion-src-045;fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
       </x:c>
       <x:c r="J35" s="31" t="str">
         <x:v>supports</x:v>
@@ -7769,7 +7964,7 @@
         <x:v>frozen_tokamak_pathway</x:v>
       </x:c>
       <x:c r="N35" s="31" t="str">
-        <x:v>matched</x:v>
+        <x:v>designed_under_development_not_completed</x:v>
       </x:c>
       <x:c r="O35" s="31" t="str">
         <x:v>missing</x:v>
@@ -7893,10 +8088,10 @@
         <x:v>inference</x:v>
       </x:c>
       <x:c r="H37" s="31" t="str">
-        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-US-NSTXU</x:v>
+        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO</x:v>
       </x:c>
       <x:c r="I37" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-012;fusion-src-014;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-012;fusion-src-014</x:v>
       </x:c>
       <x:c r="J37" s="31" t="str">
         <x:v>supports_with_limits</x:v>
@@ -7964,10 +8159,10 @@
         <x:v>observed facility milestone</x:v>
       </x:c>
       <x:c r="H38" s="31" t="str">
-        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-US-NSTXU</x:v>
+        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO</x:v>
       </x:c>
       <x:c r="I38" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-012;fusion-src-014;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-012;fusion-src-014</x:v>
       </x:c>
       <x:c r="J38" s="31" t="str">
         <x:v>supports</x:v>
@@ -8035,10 +8230,10 @@
         <x:v>inference</x:v>
       </x:c>
       <x:c r="H39" s="31" t="str">
-        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-US-NSTXU</x:v>
+        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO</x:v>
       </x:c>
       <x:c r="I39" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-012;fusion-src-014;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-012;fusion-src-014</x:v>
       </x:c>
       <x:c r="J39" s="31" t="str">
         <x:v>complicates</x:v>
@@ -8106,10 +8301,10 @@
         <x:v>observed facility milestone</x:v>
       </x:c>
       <x:c r="H40" s="31" t="str">
-        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-US-NSTXU</x:v>
+        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO</x:v>
       </x:c>
       <x:c r="I40" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-012;fusion-src-014;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-012;fusion-src-014</x:v>
       </x:c>
       <x:c r="J40" s="31" t="str">
         <x:v>supports</x:v>
@@ -8177,10 +8372,10 @@
         <x:v>inference</x:v>
       </x:c>
       <x:c r="H41" s="31" t="str">
-        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-US-NSTXU</x:v>
+        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO</x:v>
       </x:c>
       <x:c r="I41" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-012;fusion-src-014;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-012;fusion-src-014</x:v>
       </x:c>
       <x:c r="J41" s="31" t="str">
         <x:v>complicates</x:v>
@@ -9668,10 +9863,10 @@
         <x:v>inference</x:v>
       </x:c>
       <x:c r="H62" s="31" t="str">
-        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-CN-MFG;S-US-NSTXU</x:v>
+        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-CN-MFG</x:v>
       </x:c>
       <x:c r="I62" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-014;fusion-src-016;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-014;fusion-src-016</x:v>
       </x:c>
       <x:c r="J62" s="31" t="str">
         <x:v>complicates</x:v>
@@ -9739,10 +9934,10 @@
         <x:v>observed facility milestone</x:v>
       </x:c>
       <x:c r="H63" s="31" t="str">
-        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-CN-MFG;S-US-NSTXU</x:v>
+        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-CN-MFG</x:v>
       </x:c>
       <x:c r="I63" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-014;fusion-src-016;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-014;fusion-src-016</x:v>
       </x:c>
       <x:c r="J63" s="31" t="str">
         <x:v>supports</x:v>
@@ -9810,10 +10005,10 @@
         <x:v>inference</x:v>
       </x:c>
       <x:c r="H64" s="31" t="str">
-        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-CN-MFG;S-US-NSTXU</x:v>
+        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-CN-MFG</x:v>
       </x:c>
       <x:c r="I64" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-014;fusion-src-016;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-014;fusion-src-016</x:v>
       </x:c>
       <x:c r="J64" s="31" t="str">
         <x:v>complicates</x:v>
@@ -9881,10 +10076,10 @@
         <x:v>observed facility milestone</x:v>
       </x:c>
       <x:c r="H65" s="31" t="str">
-        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-CN-MFG;S-US-NSTXU</x:v>
+        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-CN-MFG</x:v>
       </x:c>
       <x:c r="I65" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-014;fusion-src-016;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-014;fusion-src-016</x:v>
       </x:c>
       <x:c r="J65" s="31" t="str">
         <x:v>supports</x:v>
@@ -9952,10 +10147,10 @@
         <x:v>observed facility milestone</x:v>
       </x:c>
       <x:c r="H66" s="31" t="str">
-        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-CN-MFG;S-US-NSTXU</x:v>
+        <x:v>S-CN-CRAFT-TF;S-CN-HH70-CO;S-CN-MFG</x:v>
       </x:c>
       <x:c r="I66" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-014;fusion-src-016;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-014;fusion-src-016</x:v>
       </x:c>
       <x:c r="J66" s="31" t="str">
         <x:v>supports</x:v>
@@ -10023,10 +10218,10 @@
         <x:v>inference</x:v>
       </x:c>
       <x:c r="H67" s="31" t="str">
-        <x:v>S-CN-CFEC;S-CN-HH70-CO;S-CN-MFG;S-JP-JT60;S-ITER-BASE</x:v>
+        <x:v>S-CN-CFEC;S-CN-HH70-CO;S-CN-MFG;S-US-NSTXU;S-JP-JT60;S-ITER-BASE;S-ITER-2026</x:v>
       </x:c>
       <x:c r="I67" s="31" t="str">
-        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-033;fusion-src-036</x:v>
+        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-030;fusion-src-033;fusion-src-036;fusion-src-037</x:v>
       </x:c>
       <x:c r="J67" s="31" t="str">
         <x:v>complicates</x:v>
@@ -10094,10 +10289,10 @@
         <x:v>programme announcement</x:v>
       </x:c>
       <x:c r="H68" s="31" t="str">
-        <x:v>S-CN-CFEC;S-CN-HH70-CO;S-CN-MFG;S-JP-JT60;S-ITER-BASE</x:v>
+        <x:v>S-CN-CFEC;S-CN-HH70-CO;S-CN-MFG;S-US-NSTXU;S-JP-JT60;S-ITER-BASE;S-ITER-2026</x:v>
       </x:c>
       <x:c r="I68" s="31" t="str">
-        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-033;fusion-src-036</x:v>
+        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-030;fusion-src-033;fusion-src-036;fusion-src-037</x:v>
       </x:c>
       <x:c r="J68" s="31" t="str">
         <x:v>supports</x:v>
@@ -10165,10 +10360,10 @@
         <x:v>inference</x:v>
       </x:c>
       <x:c r="H69" s="31" t="str">
-        <x:v>S-CN-CFEC;S-CN-HH70-CO;S-CN-MFG;S-JP-JT60;S-ITER-BASE</x:v>
+        <x:v>S-CN-CFEC;S-CN-HH70-CO;S-CN-MFG;S-US-NSTXU;S-JP-JT60;S-ITER-BASE;S-ITER-2026</x:v>
       </x:c>
       <x:c r="I69" s="31" t="str">
-        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-033;fusion-src-036</x:v>
+        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-030;fusion-src-033;fusion-src-036;fusion-src-037</x:v>
       </x:c>
       <x:c r="J69" s="31" t="str">
         <x:v>complicates</x:v>
@@ -10236,10 +10431,10 @@
         <x:v>programme announcement</x:v>
       </x:c>
       <x:c r="H70" s="31" t="str">
-        <x:v>S-CN-CFEC;S-CN-HH70-CO;S-CN-MFG;S-JP-JT60;S-ITER-BASE</x:v>
+        <x:v>S-CN-CFEC;S-CN-HH70-CO;S-CN-MFG;S-US-NSTXU;S-JP-JT60;S-ITER-BASE;S-ITER-2026</x:v>
       </x:c>
       <x:c r="I70" s="31" t="str">
-        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-033;fusion-src-036</x:v>
+        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-030;fusion-src-033;fusion-src-036;fusion-src-037</x:v>
       </x:c>
       <x:c r="J70" s="31" t="str">
         <x:v>supports</x:v>
@@ -10307,10 +10502,10 @@
         <x:v>programme announcement</x:v>
       </x:c>
       <x:c r="H71" s="31" t="str">
-        <x:v>S-CN-CFEC;S-CN-HH70-CO;S-CN-MFG;S-JP-JT60;S-ITER-BASE</x:v>
+        <x:v>S-CN-CFEC;S-CN-HH70-CO;S-CN-MFG;S-US-NSTXU;S-JP-JT60;S-ITER-BASE;S-ITER-2026</x:v>
       </x:c>
       <x:c r="I71" s="31" t="str">
-        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-033;fusion-src-036</x:v>
+        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-030;fusion-src-033;fusion-src-036;fusion-src-037</x:v>
       </x:c>
       <x:c r="J71" s="31" t="str">
         <x:v>supports</x:v>
@@ -11136,7 +11331,7 @@
         <x:v>Coverage statement only; this row does not select or recode an S value.</x:v>
       </x:c>
     </x:row>
-    <x:row r="83" ht="129.60000610351562" hidden="0" customHeight="1">
+    <x:row r="83" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A83" s="31" t="str">
         <x:v>fusion-clm-082</x:v>
       </x:c>
@@ -11150,13 +11345,13 @@
         <x:v>S2</x:v>
       </x:c>
       <x:c r="E83" s="31" t="str">
-        <x:v>The verified source set directly informs feedback speed for Licensing within the frozen research-to-pilot pathway.</x:v>
+        <x:v>The enacted-law, proposed-rule, and regulator-status sources establish legal status but do not empirically establish fusion licence-review feedback speed; the NRC rulemaking comment interval is not a plant-licence review duration.</x:v>
       </x:c>
       <x:c r="F83" s="31" t="str">
-        <x:v>programme announcement</x:v>
+        <x:v>inference</x:v>
       </x:c>
       <x:c r="G83" s="31" t="str">
-        <x:v>programme announcement</x:v>
+        <x:v>inference</x:v>
       </x:c>
       <x:c r="H83" s="31" t="str">
         <x:v>S-CN-LAW;S-US-NRC;S-IAEA-SAFE</x:v>
@@ -11165,19 +11360,19 @@
         <x:v>fusion-src-004;fusion-src-039;fusion-src-040;fusion-src-041</x:v>
       </x:c>
       <x:c r="J83" s="31" t="str">
-        <x:v>supports</x:v>
+        <x:v>complicates</x:v>
       </x:c>
       <x:c r="K83" s="31" t="str">
-        <x:v>direct</x:v>
+        <x:v>indirect</x:v>
       </x:c>
       <x:c r="L83" s="31" t="str">
-        <x:v>exact_stage</x:v>
+        <x:v>partial</x:v>
       </x:c>
       <x:c r="M83" s="31" t="str">
         <x:v>frozen_tokamak_pathway</x:v>
       </x:c>
       <x:c r="N83" s="31" t="str">
-        <x:v>matched</x:v>
+        <x:v>partial</x:v>
       </x:c>
       <x:c r="O83" s="31" t="str">
         <x:v>missing</x:v>
@@ -11221,7 +11416,7 @@
         <x:v>S3</x:v>
       </x:c>
       <x:c r="E84" s="31" t="str">
-        <x:v>A bounded first-pass search located no suitable source directly supporting a claim about experiment affordability and throughput for Licensing; this is not evidence of absence.</x:v>
+        <x:v>No suitable source in this bounded pass directly establishes the affordability or throughput of a comparable fusion pilot-plant licensing review; this is not evidence of absence.</x:v>
       </x:c>
       <x:c r="F84" s="31" t="str">
         <x:v>commentary</x:v>
@@ -11278,7 +11473,7 @@
         <x:v>Coverage statement only; this row does not select or recode an S value.</x:v>
       </x:c>
     </x:row>
-    <x:row r="85" ht="151.1999969482422" hidden="0" customHeight="1">
+    <x:row r="85" ht="226.8000030517578" hidden="0" customHeight="1">
       <x:c r="A85" s="31" t="str">
         <x:v>fusion-clm-084</x:v>
       </x:c>
@@ -11292,13 +11487,13 @@
         <x:v>S4</x:v>
       </x:c>
       <x:c r="E85" s="31" t="str">
-        <x:v>The verified source set directly informs physical flexibility or elapsed-time floors for Licensing within the frozen research-to-pilot pathway.</x:v>
+        <x:v>The legal and regulatory sources provide at most indirect, partial evidence about licensing elapsed-time floors; they do not empirically prove that licensing lacks an intrinsic process constraint.</x:v>
       </x:c>
       <x:c r="F85" s="31" t="str">
-        <x:v>programme announcement</x:v>
+        <x:v>inference</x:v>
       </x:c>
       <x:c r="G85" s="31" t="str">
-        <x:v>programme announcement</x:v>
+        <x:v>inference</x:v>
       </x:c>
       <x:c r="H85" s="31" t="str">
         <x:v>S-CN-LAW;S-US-NRC;S-IAEA-SAFE</x:v>
@@ -11307,19 +11502,19 @@
         <x:v>fusion-src-004;fusion-src-039;fusion-src-040;fusion-src-041</x:v>
       </x:c>
       <x:c r="J85" s="31" t="str">
-        <x:v>supports</x:v>
+        <x:v>supports_with_limits</x:v>
       </x:c>
       <x:c r="K85" s="31" t="str">
-        <x:v>direct</x:v>
+        <x:v>indirect</x:v>
       </x:c>
       <x:c r="L85" s="31" t="str">
-        <x:v>exact_stage</x:v>
+        <x:v>partial</x:v>
       </x:c>
       <x:c r="M85" s="31" t="str">
         <x:v>frozen_tokamak_pathway</x:v>
       </x:c>
       <x:c r="N85" s="31" t="str">
-        <x:v>matched</x:v>
+        <x:v>partial</x:v>
       </x:c>
       <x:c r="O85" s="31" t="str">
         <x:v>missing</x:v>
@@ -11349,7 +11544,7 @@
         <x:v>Coverage statement only; this row does not select or recode an S value.</x:v>
       </x:c>
     </x:row>
-    <x:row r="86" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="86" ht="205.1999969482422" hidden="0" customHeight="1">
       <x:c r="A86" s="31" t="str">
         <x:v>fusion-clm-085</x:v>
       </x:c>
@@ -11363,7 +11558,7 @@
         <x:v>S5</x:v>
       </x:c>
       <x:c r="E86" s="31" t="str">
-        <x:v>The verified source set informs intrinsic error tolerance for Licensing only by bounded analogy or adjacent-stage evidence.</x:v>
+        <x:v>The legal and regulatory sources inform licensing error tolerance only indirectly and remain domain-sensitive; no completed comparable fusion licence case resolves the issue.</x:v>
       </x:c>
       <x:c r="F86" s="31" t="str">
         <x:v>inference</x:v>
@@ -12343,7 +12538,7 @@
         <x:v>Atomic numerical or status claim; no S value is selected.</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" ht="86.4000015258789" hidden="0" customHeight="1">
+    <x:row r="100" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A100" s="31" t="str">
         <x:v>fusion-clm-099</x:v>
       </x:c>
@@ -12360,10 +12555,10 @@
         <x:v>The NRC proposed rule opened a 90-day public-comment period ending 27 May 2026.</x:v>
       </x:c>
       <x:c r="F100" s="31" t="str">
-        <x:v>programme announcement</x:v>
+        <x:v>observed legal/regulatory status</x:v>
       </x:c>
       <x:c r="G100" s="31" t="str">
-        <x:v>programme announcement</x:v>
+        <x:v>observed legal/regulatory status</x:v>
       </x:c>
       <x:c r="H100" s="31" t="str">
         <x:v>S-US-NRC</x:v>
@@ -12372,13 +12567,13 @@
         <x:v>fusion-src-039</x:v>
       </x:c>
       <x:c r="J100" s="31" t="str">
-        <x:v>supports_with_limits</x:v>
+        <x:v>complicates</x:v>
       </x:c>
       <x:c r="K100" s="31" t="str">
         <x:v>direct</x:v>
       </x:c>
       <x:c r="L100" s="31" t="str">
-        <x:v>exact_stage</x:v>
+        <x:v>partial</x:v>
       </x:c>
       <x:c r="M100" s="31" t="str">
         <x:v>frozen_tokamak_pathway</x:v>
@@ -12393,7 +12588,7 @@
         <x:v>days</x:v>
       </x:c>
       <x:c r="Q100" s="31" t="str">
-        <x:v>public-comment period</x:v>
+        <x:v>rulemaking public-comment period; not a plant-licence review</x:v>
       </x:c>
       <x:c r="R100" s="31" t="str">
         <x:v>2026-02-26 to 2026-05-27</x:v>
@@ -12402,7 +12597,7 @@
         <x:v>Federal Register Dates section.</x:v>
       </x:c>
       <x:c r="T100" s="31" t="str">
-        <x:v>Rulemaking interval is not a plant-licence review duration.</x:v>
+        <x:v>Rulemaking interval is not a plant-licence review duration and cannot support a licensing-feedback-speed estimate.</x:v>
       </x:c>
       <x:c r="U100" s="31" t="str">
         <x:v>verified_against_original</x:v>
@@ -12485,10 +12680,649 @@
         <x:v>Atomic numerical or status claim; no S value is selected.</x:v>
       </x:c>
     </x:row>
+    <x:row r="102" ht="151.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A102" s="31" t="str">
+        <x:v>fusion-clm-101</x:v>
+      </x:c>
+      <x:c r="B102" s="31" t="str">
+        <x:v>sp-0015</x:v>
+      </x:c>
+      <x:c r="C102" s="31" t="str">
+        <x:v>simulation</x:v>
+      </x:c>
+      <x:c r="D102" s="31" t="str">
+        <x:v>S2</x:v>
+      </x:c>
+      <x:c r="E102" s="31" t="str">
+        <x:v>A conventional HEAT magnetic-shadow calculation could take around 30 minutes for one simulation and longer for complex geometries.</x:v>
+      </x:c>
+      <x:c r="F102" s="31" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="G102" s="31" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="H102" s="31" t="str">
+        <x:v>unassigned_pack_table</x:v>
+      </x:c>
+      <x:c r="I102" s="31" t="str">
+        <x:v>fusion-src-023</x:v>
+      </x:c>
+      <x:c r="J102" s="31" t="str">
+        <x:v>supports_with_limits</x:v>
+      </x:c>
+      <x:c r="K102" s="31" t="str">
+        <x:v>direct</x:v>
+      </x:c>
+      <x:c r="L102" s="31" t="str">
+        <x:v>exact_stage</x:v>
+      </x:c>
+      <x:c r="M102" s="31" t="str">
+        <x:v>frozen_tokamak_pathway</x:v>
+      </x:c>
+      <x:c r="N102" s="31" t="str">
+        <x:v>geometry_specific_simulation</x:v>
+      </x:c>
+      <x:c r="O102" s="31" t="str">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="P102" s="31" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="Q102" s="31" t="str">
+        <x:v>one SPARC magnetic-shadow simulation</x:v>
+      </x:c>
+      <x:c r="R102" s="31" t="str">
+        <x:v>published 2025-08-13</x:v>
+      </x:c>
+      <x:c r="S102" s="31" t="str">
+        <x:v>PPPL article paragraph 101.</x:v>
+      </x:c>
+      <x:c r="T102" s="31" t="str">
+        <x:v>Calculation time for a small geometry-specific design task is not plant schedule or materials-qualification duration.</x:v>
+      </x:c>
+      <x:c r="U102" s="31" t="str">
+        <x:v>verified_against_original</x:v>
+      </x:c>
+      <x:c r="V102" s="31" t="str">
+        <x:v>routine_domain_review_no_owner_action</x:v>
+      </x:c>
+      <x:c r="W102" s="31" t="str">
+        <x:v>Atomic numerical or status claim; no S value is selected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A103" s="31" t="str">
+        <x:v>fusion-clm-102</x:v>
+      </x:c>
+      <x:c r="B103" s="31" t="str">
+        <x:v>sp-0015</x:v>
+      </x:c>
+      <x:c r="C103" s="31" t="str">
+        <x:v>simulation</x:v>
+      </x:c>
+      <x:c r="D103" s="31" t="str">
+        <x:v>S2</x:v>
+      </x:c>
+      <x:c r="E103" s="31" t="str">
+        <x:v>HEAT-ML reduced the scoped magnetic-shadow calculation to a few milliseconds.</x:v>
+      </x:c>
+      <x:c r="F103" s="31" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="G103" s="31" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="H103" s="31" t="str">
+        <x:v>unassigned_pack_table</x:v>
+      </x:c>
+      <x:c r="I103" s="31" t="str">
+        <x:v>fusion-src-023</x:v>
+      </x:c>
+      <x:c r="J103" s="31" t="str">
+        <x:v>supports_with_limits</x:v>
+      </x:c>
+      <x:c r="K103" s="31" t="str">
+        <x:v>direct</x:v>
+      </x:c>
+      <x:c r="L103" s="31" t="str">
+        <x:v>exact_stage</x:v>
+      </x:c>
+      <x:c r="M103" s="31" t="str">
+        <x:v>frozen_tokamak_pathway</x:v>
+      </x:c>
+      <x:c r="N103" s="31" t="str">
+        <x:v>geometry_specific_simulation</x:v>
+      </x:c>
+      <x:c r="O103" s="31" t="str">
+        <x:v>few</x:v>
+      </x:c>
+      <x:c r="P103" s="31" t="str">
+        <x:v>milliseconds</x:v>
+      </x:c>
+      <x:c r="Q103" s="31" t="str">
+        <x:v>one SPARC magnetic-shadow calculation</x:v>
+      </x:c>
+      <x:c r="R103" s="31" t="str">
+        <x:v>published 2025-08-13</x:v>
+      </x:c>
+      <x:c r="S103" s="31" t="str">
+        <x:v>PPPL article paragraph 102; linked DOI 10.1016/j.fusengdes.2025.115010.</x:v>
+      </x:c>
+      <x:c r="T103" s="31" t="str">
+        <x:v>The method is tied to 15 tiles in a small part of SPARC's exhaust geometry; no plant-level acceleration is established.</x:v>
+      </x:c>
+      <x:c r="U103" s="31" t="str">
+        <x:v>verified_against_original</x:v>
+      </x:c>
+      <x:c r="V103" s="31" t="str">
+        <x:v>routine_domain_review_no_owner_action</x:v>
+      </x:c>
+      <x:c r="W103" s="31" t="str">
+        <x:v>Atomic numerical or status claim; no S value is selected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104" ht="129.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A104" s="31" t="str">
+        <x:v>fusion-clm-103</x:v>
+      </x:c>
+      <x:c r="B104" s="31" t="str">
+        <x:v>sp-0015</x:v>
+      </x:c>
+      <x:c r="C104" s="31" t="str">
+        <x:v>simulation</x:v>
+      </x:c>
+      <x:c r="D104" s="31" t="str">
+        <x:v>S3</x:v>
+      </x:c>
+      <x:c r="E104" s="31" t="str">
+        <x:v>The HEAT-ML neural network used a training database of approximately 1,000 SPARC HEAT simulations.</x:v>
+      </x:c>
+      <x:c r="F104" s="31" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="G104" s="31" t="str">
+        <x:v>proof of concept</x:v>
+      </x:c>
+      <x:c r="H104" s="31" t="str">
+        <x:v>unassigned_pack_table</x:v>
+      </x:c>
+      <x:c r="I104" s="31" t="str">
+        <x:v>fusion-src-023</x:v>
+      </x:c>
+      <x:c r="J104" s="31" t="str">
+        <x:v>supports_with_limits</x:v>
+      </x:c>
+      <x:c r="K104" s="31" t="str">
+        <x:v>direct</x:v>
+      </x:c>
+      <x:c r="L104" s="31" t="str">
+        <x:v>exact_stage</x:v>
+      </x:c>
+      <x:c r="M104" s="31" t="str">
+        <x:v>frozen_tokamak_pathway</x:v>
+      </x:c>
+      <x:c r="N104" s="31" t="str">
+        <x:v>geometry_specific_simulation</x:v>
+      </x:c>
+      <x:c r="O104" s="31" t="str">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="P104" s="31" t="str">
+        <x:v>simulations</x:v>
+      </x:c>
+      <x:c r="Q104" s="31" t="str">
+        <x:v>approximately; SPARC HEAT training database</x:v>
+      </x:c>
+      <x:c r="R104" s="31" t="str">
+        <x:v>published 2025-08-13</x:v>
+      </x:c>
+      <x:c r="S104" s="31" t="str">
+        <x:v>PPPL article paragraph 102.</x:v>
+      </x:c>
+      <x:c r="T104" s="31" t="str">
+        <x:v>Training-set size is not an affordability, qualification-throughput, or generic plasma-facing-component outcome.</x:v>
+      </x:c>
+      <x:c r="U104" s="31" t="str">
+        <x:v>verified_against_original</x:v>
+      </x:c>
+      <x:c r="V104" s="31" t="str">
+        <x:v>routine_domain_review_no_owner_action</x:v>
+      </x:c>
+      <x:c r="W104" s="31" t="str">
+        <x:v>Atomic numerical or status claim; no S value is selected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105" ht="140.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A105" s="31" t="str">
+        <x:v>fusion-clm-104</x:v>
+      </x:c>
+      <x:c r="B105" s="31" t="str">
+        <x:v>sp-0027</x:v>
+      </x:c>
+      <x:c r="C105" s="31" t="str">
+        <x:v>construction</x:v>
+      </x:c>
+      <x:c r="D105" s="31" t="str">
+        <x:v>S4</x:v>
+      </x:c>
+      <x:c r="E105" s="31" t="str">
+        <x:v>ITER installed the sixth of nine tokamak sector modules during 27-28 July 2026, putting two-thirds of the plasma chamber in place.</x:v>
+      </x:c>
+      <x:c r="F105" s="31" t="str">
+        <x:v>observed facility milestone</x:v>
+      </x:c>
+      <x:c r="G105" s="31" t="str">
+        <x:v>observed facility milestone</x:v>
+      </x:c>
+      <x:c r="H105" s="31" t="str">
+        <x:v>S-ITER-2026</x:v>
+      </x:c>
+      <x:c r="I105" s="31" t="str">
+        <x:v>fusion-src-037</x:v>
+      </x:c>
+      <x:c r="J105" s="31" t="str">
+        <x:v>supports_with_limits</x:v>
+      </x:c>
+      <x:c r="K105" s="31" t="str">
+        <x:v>direct</x:v>
+      </x:c>
+      <x:c r="L105" s="31" t="str">
+        <x:v>exact_stage</x:v>
+      </x:c>
+      <x:c r="M105" s="31" t="str">
+        <x:v>frozen_tokamak_pathway</x:v>
+      </x:c>
+      <x:c r="N105" s="31" t="str">
+        <x:v>construction_not_completion</x:v>
+      </x:c>
+      <x:c r="O105" s="31" t="str">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="P105" s="31" t="str">
+        <x:v>sector modules</x:v>
+      </x:c>
+      <x:c r="Q105" s="31" t="str">
+        <x:v>nine-module plasma chamber; two-thirds installed</x:v>
+      </x:c>
+      <x:c r="R105" s="31" t="str">
+        <x:v>2026-07-27 to 2026-07-28</x:v>
+      </x:c>
+      <x:c r="S105" s="31" t="str">
+        <x:v>ITER article paragraphs 162 and 167; official road-to-ITER milestone page.</x:v>
+      </x:c>
+      <x:c r="T105" s="31" t="str">
+        <x:v>Observed construction milestone only; not an AI result, completed chamber, commissioning, or plant completion.</x:v>
+      </x:c>
+      <x:c r="U105" s="31" t="str">
+        <x:v>verified_against_original</x:v>
+      </x:c>
+      <x:c r="V105" s="31" t="str">
+        <x:v>routine_domain_review_no_owner_action</x:v>
+      </x:c>
+      <x:c r="W105" s="31" t="str">
+        <x:v>Atomic numerical or status claim; no S value is selected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="106" ht="140.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A106" s="31" t="str">
+        <x:v>fusion-clm-105</x:v>
+      </x:c>
+      <x:c r="B106" s="31" t="str">
+        <x:v>sp-0028</x:v>
+      </x:c>
+      <x:c r="C106" s="31" t="str">
+        <x:v>commissioning</x:v>
+      </x:c>
+      <x:c r="D106" s="31" t="str">
+        <x:v>S4</x:v>
+      </x:c>
+      <x:c r="E106" s="31" t="str">
+        <x:v>PPPL's living NSTX-U page stated that the Recovery Project was 93% complete when checked on 31 August 2026.</x:v>
+      </x:c>
+      <x:c r="F106" s="31" t="str">
+        <x:v>observed facility milestone</x:v>
+      </x:c>
+      <x:c r="G106" s="31" t="str">
+        <x:v>observed facility milestone</x:v>
+      </x:c>
+      <x:c r="H106" s="31" t="str">
+        <x:v>S-US-NSTXU</x:v>
+      </x:c>
+      <x:c r="I106" s="31" t="str">
+        <x:v>fusion-src-030</x:v>
+      </x:c>
+      <x:c r="J106" s="31" t="str">
+        <x:v>supports_with_limits</x:v>
+      </x:c>
+      <x:c r="K106" s="31" t="str">
+        <x:v>direct</x:v>
+      </x:c>
+      <x:c r="L106" s="31" t="str">
+        <x:v>partial</x:v>
+      </x:c>
+      <x:c r="M106" s="31" t="str">
+        <x:v>frozen_tokamak_pathway</x:v>
+      </x:c>
+      <x:c r="N106" s="31" t="str">
+        <x:v>living_project_status_not_recommissioning</x:v>
+      </x:c>
+      <x:c r="O106" s="31" t="str">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="P106" s="31" t="str">
+        <x:v>percent</x:v>
+      </x:c>
+      <x:c r="Q106" s="31" t="str">
+        <x:v>NSTX-U Recovery Project status on a mutable living page</x:v>
+      </x:c>
+      <x:c r="R106" s="31" t="str">
+        <x:v>checked 2026-08-31</x:v>
+      </x:c>
+      <x:c r="S106" s="31" t="str">
+        <x:v>PPPL NSTX-U page, section 'Recovery Project'.</x:v>
+      </x:c>
+      <x:c r="T106" s="31" t="str">
+        <x:v>Not completed recommissioning, a fixed historical statistic, or an experimental outcome; recheck on any project-page update.</x:v>
+      </x:c>
+      <x:c r="U106" s="31" t="str">
+        <x:v>verified_against_original</x:v>
+      </x:c>
+      <x:c r="V106" s="31" t="str">
+        <x:v>routine_domain_review_no_owner_action</x:v>
+      </x:c>
+      <x:c r="W106" s="31" t="str">
+        <x:v>Atomic numerical or status claim; no S value is selected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107" ht="129.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A107" s="31" t="str">
+        <x:v>fusion-clm-106</x:v>
+      </x:c>
+      <x:c r="B107" s="31" t="str">
+        <x:v>sp-0020</x:v>
+      </x:c>
+      <x:c r="C107" s="31" t="str">
+        <x:v>materials_qualification</x:v>
+      </x:c>
+      <x:c r="D107" s="31" t="str">
+        <x:v>S2</x:v>
+      </x:c>
+      <x:c r="E107" s="31" t="str">
+        <x:v>IFMIF-DONES targets roughly 20-30 dpa over about 2.5 full-power years in approximately 300 cm3.</x:v>
+      </x:c>
+      <x:c r="F107" s="31" t="str">
+        <x:v>official target</x:v>
+      </x:c>
+      <x:c r="G107" s="31" t="str">
+        <x:v>official target</x:v>
+      </x:c>
+      <x:c r="H107" s="31" t="str">
+        <x:v>targeted_ifmif_dones</x:v>
+      </x:c>
+      <x:c r="I107" s="31" t="str">
+        <x:v>fusion-src-046</x:v>
+      </x:c>
+      <x:c r="J107" s="31" t="str">
+        <x:v>supports_with_limits</x:v>
+      </x:c>
+      <x:c r="K107" s="31" t="str">
+        <x:v>direct</x:v>
+      </x:c>
+      <x:c r="L107" s="31" t="str">
+        <x:v>exact_stage</x:v>
+      </x:c>
+      <x:c r="M107" s="31" t="str">
+        <x:v>frozen_tokamak_pathway</x:v>
+      </x:c>
+      <x:c r="N107" s="31" t="str">
+        <x:v>designed_under_development_not_completed</x:v>
+      </x:c>
+      <x:c r="O107" s="31" t="str">
+        <x:v>20-30</x:v>
+      </x:c>
+      <x:c r="P107" s="31" t="str">
+        <x:v>dpa</x:v>
+      </x:c>
+      <x:c r="Q107" s="31" t="str">
+        <x:v>approximately 300 cm3 high-flux volume</x:v>
+      </x:c>
+      <x:c r="R107" s="31" t="str">
+        <x:v>about 2.5 full-power years</x:v>
+      </x:c>
+      <x:c r="S107" s="31" t="str">
+        <x:v>IAEA technical-meeting contribution, Description paragraph 2.</x:v>
+      </x:c>
+      <x:c r="T107" s="31" t="str">
+        <x:v>Accelerator-driven fusion-like neutron exposure target; not an observed campaign or completed accepted qualification dataset.</x:v>
+      </x:c>
+      <x:c r="U107" s="31" t="str">
+        <x:v>verified_against_original</x:v>
+      </x:c>
+      <x:c r="V107" s="31" t="str">
+        <x:v>routine_domain_review_no_owner_action</x:v>
+      </x:c>
+      <x:c r="W107" s="31" t="str">
+        <x:v>Atomic numerical or status claim; no S value is selected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="108" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A108" s="31" t="str">
+        <x:v>fusion-clm-107</x:v>
+      </x:c>
+      <x:c r="B108" s="31" t="str">
+        <x:v>sp-0020</x:v>
+      </x:c>
+      <x:c r="C108" s="31" t="str">
+        <x:v>materials_qualification</x:v>
+      </x:c>
+      <x:c r="D108" s="31" t="str">
+        <x:v>S2</x:v>
+      </x:c>
+      <x:c r="E108" s="31" t="str">
+        <x:v>IFMIF-DONES targets 50 dpa in about 3 full-power years in approximately 100 cm3.</x:v>
+      </x:c>
+      <x:c r="F108" s="31" t="str">
+        <x:v>official target</x:v>
+      </x:c>
+      <x:c r="G108" s="31" t="str">
+        <x:v>official target</x:v>
+      </x:c>
+      <x:c r="H108" s="31" t="str">
+        <x:v>targeted_ifmif_dones</x:v>
+      </x:c>
+      <x:c r="I108" s="31" t="str">
+        <x:v>fusion-src-045;fusion-src-046</x:v>
+      </x:c>
+      <x:c r="J108" s="31" t="str">
+        <x:v>supports_with_limits</x:v>
+      </x:c>
+      <x:c r="K108" s="31" t="str">
+        <x:v>direct</x:v>
+      </x:c>
+      <x:c r="L108" s="31" t="str">
+        <x:v>exact_stage</x:v>
+      </x:c>
+      <x:c r="M108" s="31" t="str">
+        <x:v>frozen_tokamak_pathway</x:v>
+      </x:c>
+      <x:c r="N108" s="31" t="str">
+        <x:v>designed_under_development_not_completed</x:v>
+      </x:c>
+      <x:c r="O108" s="31" t="str">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="P108" s="31" t="str">
+        <x:v>dpa</x:v>
+      </x:c>
+      <x:c r="Q108" s="31" t="str">
+        <x:v>approximately 100 cm3 high-flux volume</x:v>
+      </x:c>
+      <x:c r="R108" s="31" t="str">
+        <x:v>about 3 full-power years</x:v>
+      </x:c>
+      <x:c r="S108" s="31" t="str">
+        <x:v>IAEA contribution Description paragraph 2; peer-reviewed paper HFTM section, DOI 10.1088/1741-4326/add172.</x:v>
+      </x:c>
+      <x:c r="T108" s="31" t="str">
+        <x:v>A designed irradiation target directly supports a physical time floor but is not a completed dataset.</x:v>
+      </x:c>
+      <x:c r="U108" s="31" t="str">
+        <x:v>verified_against_original</x:v>
+      </x:c>
+      <x:c r="V108" s="31" t="str">
+        <x:v>routine_domain_review_no_owner_action</x:v>
+      </x:c>
+      <x:c r="W108" s="31" t="str">
+        <x:v>Atomic numerical or status claim; no S value is selected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="109" ht="140.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A109" s="31" t="str">
+        <x:v>fusion-clm-108</x:v>
+      </x:c>
+      <x:c r="B109" s="31" t="str">
+        <x:v>sp-0020</x:v>
+      </x:c>
+      <x:c r="C109" s="31" t="str">
+        <x:v>materials_qualification</x:v>
+      </x:c>
+      <x:c r="D109" s="31" t="str">
+        <x:v>S4</x:v>
+      </x:c>
+      <x:c r="E109" s="31" t="str">
+        <x:v>The IFMIF-DONES qualification chain includes post-irradiation examination after the multi-year HFTM campaign.</x:v>
+      </x:c>
+      <x:c r="F109" s="31" t="str">
+        <x:v>model or scenario estimate</x:v>
+      </x:c>
+      <x:c r="G109" s="31" t="str">
+        <x:v>model or scenario estimate</x:v>
+      </x:c>
+      <x:c r="H109" s="31" t="str">
+        <x:v>targeted_ifmif_dones</x:v>
+      </x:c>
+      <x:c r="I109" s="31" t="str">
+        <x:v>fusion-src-045</x:v>
+      </x:c>
+      <x:c r="J109" s="31" t="str">
+        <x:v>supports_with_limits</x:v>
+      </x:c>
+      <x:c r="K109" s="31" t="str">
+        <x:v>direct</x:v>
+      </x:c>
+      <x:c r="L109" s="31" t="str">
+        <x:v>exact_stage</x:v>
+      </x:c>
+      <x:c r="M109" s="31" t="str">
+        <x:v>frozen_tokamak_pathway</x:v>
+      </x:c>
+      <x:c r="N109" s="31" t="str">
+        <x:v>designed_under_development_not_completed</x:v>
+      </x:c>
+      <x:c r="O109" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="P109" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="Q109" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="R109" s="31" t="str">
+        <x:v>future programme</x:v>
+      </x:c>
+      <x:c r="S109" s="31" t="str">
+        <x:v>Peer-reviewed paper discussion of post-irradiation tests and TRTM PIE; DOI 10.1088/1741-4326/add172.</x:v>
+      </x:c>
+      <x:c r="T109" s="31" t="str">
+        <x:v>Irradiation duration does not exhaust the qualification timeline; examination and acceptance remain downstream.</x:v>
+      </x:c>
+      <x:c r="U109" s="31" t="str">
+        <x:v>verified_against_original</x:v>
+      </x:c>
+      <x:c r="V109" s="31" t="str">
+        <x:v>routine_domain_review_no_owner_action</x:v>
+      </x:c>
+      <x:c r="W109" s="31" t="str">
+        <x:v>Atomic numerical or status claim; no S value is selected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110" ht="172.8000030517578" hidden="0" customHeight="1">
+      <x:c r="A110" s="31" t="str">
+        <x:v>fusion-clm-109</x:v>
+      </x:c>
+      <x:c r="B110" s="31" t="str">
+        <x:v>sp-0020</x:v>
+      </x:c>
+      <x:c r="C110" s="31" t="str">
+        <x:v>materials_qualification</x:v>
+      </x:c>
+      <x:c r="D110" s="31" t="str">
+        <x:v>S3</x:v>
+      </x:c>
+      <x:c r="E110" s="31" t="str">
+        <x:v>IFMIF-DONES material and transmutation matching varies by material: the HFTM is tailored to Eurofer, while tungsten and copper conditions are not perfectly matched.</x:v>
+      </x:c>
+      <x:c r="F110" s="31" t="str">
+        <x:v>model or scenario estimate</x:v>
+      </x:c>
+      <x:c r="G110" s="31" t="str">
+        <x:v>model or scenario estimate</x:v>
+      </x:c>
+      <x:c r="H110" s="31" t="str">
+        <x:v>targeted_ifmif_dones</x:v>
+      </x:c>
+      <x:c r="I110" s="31" t="str">
+        <x:v>fusion-src-045</x:v>
+      </x:c>
+      <x:c r="J110" s="31" t="str">
+        <x:v>complicates</x:v>
+      </x:c>
+      <x:c r="K110" s="31" t="str">
+        <x:v>direct</x:v>
+      </x:c>
+      <x:c r="L110" s="31" t="str">
+        <x:v>exact_stage</x:v>
+      </x:c>
+      <x:c r="M110" s="31" t="str">
+        <x:v>frozen_tokamak_pathway</x:v>
+      </x:c>
+      <x:c r="N110" s="31" t="str">
+        <x:v>material_specific_transfer</x:v>
+      </x:c>
+      <x:c r="O110" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="P110" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="Q110" s="31" t="str">
+        <x:v>missing</x:v>
+      </x:c>
+      <x:c r="R110" s="31" t="str">
+        <x:v>facility design</x:v>
+      </x:c>
+      <x:c r="S110" s="31" t="str">
+        <x:v>Peer-reviewed paper Introduction/HFTM discussion; DOI 10.1088/1741-4326/add172.</x:v>
+      </x:c>
+      <x:c r="T110" s="31" t="str">
+        <x:v>Do not generalize one material's dpa and transmutation match to all fusion-grade materials.</x:v>
+      </x:c>
+      <x:c r="U110" s="31" t="str">
+        <x:v>verified_against_original</x:v>
+      </x:c>
+      <x:c r="V110" s="31" t="str">
+        <x:v>routine_domain_review_no_owner_action</x:v>
+      </x:c>
+      <x:c r="W110" s="31" t="str">
+        <x:v>Atomic numerical or status claim; no S value is selected.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5b1a667fcc84a49"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf9646bf02504ec0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12781,7 +13615,7 @@
         <x:v>The verified source set directly informs information intensity for Simulation within the frozen research-to-pilot pathway.</x:v>
       </x:c>
       <x:c r="I3" s="31" t="str">
-        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-024</x:v>
+        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-023;fusion-src-024</x:v>
       </x:c>
       <x:c r="J3" s="31" t="str">
         <x:v>peer-reviewed proof of concept plus programme evidence</x:v>
@@ -12799,7 +13633,7 @@
         <x:v>The verified source set informs feedback speed for Simulation only by bounded analogy or adjacent-stage evidence.</x:v>
       </x:c>
       <x:c r="O3" s="31" t="str">
-        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-024</x:v>
+        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-023;fusion-src-024</x:v>
       </x:c>
       <x:c r="P3" s="31" t="str">
         <x:v>peer-reviewed proof of concept plus programme evidence</x:v>
@@ -12817,7 +13651,7 @@
         <x:v>The verified source set informs experiment affordability and throughput for Simulation only by bounded analogy or adjacent-stage evidence.</x:v>
       </x:c>
       <x:c r="U3" s="31" t="str">
-        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-024</x:v>
+        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-023;fusion-src-024</x:v>
       </x:c>
       <x:c r="V3" s="31" t="str">
         <x:v>peer-reviewed proof of concept plus programme evidence</x:v>
@@ -12835,7 +13669,7 @@
         <x:v>The verified source set complicates any simple claim about physical flexibility or elapsed-time floors for Simulation; physical scope and lifecycle distinctions remain load-bearing.</x:v>
       </x:c>
       <x:c r="AA3" s="31" t="str">
-        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-024</x:v>
+        <x:v>fusion-src-007;fusion-src-017;fusion-src-022;fusion-src-023;fusion-src-024</x:v>
       </x:c>
       <x:c r="AB3" s="31" t="str">
         <x:v>peer-reviewed proof of concept plus programme evidence</x:v>
@@ -13305,7 +14139,7 @@
         <x:v>targeted_primary_source_search_only_if_load_bearing</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="183.60000610351562" hidden="0" customHeight="1">
+    <x:row r="8" ht="237.60000610351562" hidden="0" customHeight="1">
       <x:c r="A8" s="31" t="str">
         <x:v>sp-0020</x:v>
       </x:c>
@@ -13331,10 +14165,10 @@
         <x:v>The verified source set informs information intensity for Materials qualification only by bounded analogy or adjacent-stage evidence.</x:v>
       </x:c>
       <x:c r="I8" s="31" t="str">
-        <x:v>fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
+        <x:v>fusion-src-046;fusion-src-045;fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
       </x:c>
       <x:c r="J8" s="31" t="str">
-        <x:v>official requirements and planned facilities; no completed qualification case</x:v>
+        <x:v>peer-reviewed design and official programme targets; no completed accepted qualification dataset</x:v>
       </x:c>
       <x:c r="K8" s="31" t="str">
         <x:v>only_adjacent_stage_or_pathway_evidence_located</x:v>
@@ -13343,52 +14177,52 @@
         <x:v>seek_stage_and_lifecycle_matched_primary_evidence</x:v>
       </x:c>
       <x:c r="M8" s="31" t="str">
-        <x:v>contradicted or complicated</x:v>
+        <x:v>directly supported</x:v>
       </x:c>
       <x:c r="N8" s="31" t="str">
-        <x:v>The verified source set complicates any simple claim about feedback speed for Materials qualification; physical scope and lifecycle distinctions remain load-bearing.</x:v>
+        <x:v>IFMIF-DONES design and programme-target sources directly establish a planned multi-year irradiation-and-post-irradiation-examination feedback chain for materials qualification; they do not report a completed dataset.</x:v>
       </x:c>
       <x:c r="O8" s="31" t="str">
-        <x:v>fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
+        <x:v>fusion-src-046;fusion-src-045;fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
       </x:c>
       <x:c r="P8" s="31" t="str">
-        <x:v>official requirements and planned facilities; no completed qualification case</x:v>
+        <x:v>peer-reviewed design and official programme targets; no completed accepted qualification dataset</x:v>
       </x:c>
       <x:c r="Q8" s="31" t="str">
-        <x:v>available_evidence_does_not_resolve_scope_or_lifecycle_confounds</x:v>
+        <x:v>not_missing</x:v>
       </x:c>
       <x:c r="R8" s="31" t="str">
         <x:v>owner_promotion_scope_exception</x:v>
       </x:c>
       <x:c r="S8" s="31" t="str">
-        <x:v>contradicted or complicated</x:v>
+        <x:v>indirectly supported/analogy</x:v>
       </x:c>
       <x:c r="T8" s="31" t="str">
-        <x:v>The verified source set complicates any simple claim about experiment affordability and throughput for Materials qualification; physical scope and lifecycle distinctions remain load-bearing.</x:v>
+        <x:v>IFMIF-DONES planned irradiation volumes and modular campaigns inform qualification throughput only indirectly; they do not establish observed affordability, completed throughput, or acceptance.</x:v>
       </x:c>
       <x:c r="U8" s="31" t="str">
-        <x:v>fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
+        <x:v>fusion-src-046;fusion-src-045;fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
       </x:c>
       <x:c r="V8" s="31" t="str">
-        <x:v>official requirements and planned facilities; no completed qualification case</x:v>
+        <x:v>peer-reviewed design and official programme targets; no completed accepted qualification dataset</x:v>
       </x:c>
       <x:c r="W8" s="31" t="str">
-        <x:v>available_evidence_does_not_resolve_scope_or_lifecycle_confounds</x:v>
+        <x:v>only_adjacent_stage_or_pathway_evidence_located</x:v>
       </x:c>
       <x:c r="X8" s="31" t="str">
-        <x:v>preserve_complication_for_domain_review</x:v>
+        <x:v>seek_stage_and_lifecycle_matched_primary_evidence</x:v>
       </x:c>
       <x:c r="Y8" s="31" t="str">
         <x:v>directly supported</x:v>
       </x:c>
       <x:c r="Z8" s="31" t="str">
-        <x:v>The verified source set directly informs physical flexibility or elapsed-time floors for Materials qualification within the frozen research-to-pilot pathway.</x:v>
+        <x:v>IFMIF-DONES design and programme-target sources directly support a substantial physical materials-qualification time floor: roughly 2.5-3 full-power years of irradiation before the remaining examination and acceptance chain.</x:v>
       </x:c>
       <x:c r="AA8" s="31" t="str">
-        <x:v>fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
+        <x:v>fusion-src-046;fusion-src-045;fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038</x:v>
       </x:c>
       <x:c r="AB8" s="31" t="str">
-        <x:v>official requirements and planned facilities; no completed qualification case</x:v>
+        <x:v>peer-reviewed design and official programme targets; no completed accepted qualification dataset</x:v>
       </x:c>
       <x:c r="AC8" s="31" t="str">
         <x:v>not_missing</x:v>
@@ -13406,7 +14240,7 @@
         <x:v>missing</x:v>
       </x:c>
       <x:c r="AH8" s="31" t="str">
-        <x:v>official requirements and planned facilities; no completed qualification case</x:v>
+        <x:v>peer-reviewed design and official programme targets; no completed accepted qualification dataset</x:v>
       </x:c>
       <x:c r="AI8" s="31" t="str">
         <x:v>bounded_search_no_suitable_source_located_not_evidence_of_absence</x:v>
@@ -13441,7 +14275,7 @@
         <x:v>The verified source set informs information intensity for Magnets only by bounded analogy or adjacent-stage evidence.</x:v>
       </x:c>
       <x:c r="I9" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-012;fusion-src-014;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-012;fusion-src-014</x:v>
       </x:c>
       <x:c r="J9" s="31" t="str">
         <x:v>observed component/facility milestones with scope limits</x:v>
@@ -13459,7 +14293,7 @@
         <x:v>The verified source set directly informs feedback speed for Magnets within the frozen research-to-pilot pathway.</x:v>
       </x:c>
       <x:c r="O9" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-012;fusion-src-014;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-012;fusion-src-014</x:v>
       </x:c>
       <x:c r="P9" s="31" t="str">
         <x:v>observed component/facility milestones with scope limits</x:v>
@@ -13477,7 +14311,7 @@
         <x:v>The verified source set complicates any simple claim about experiment affordability and throughput for Magnets; physical scope and lifecycle distinctions remain load-bearing.</x:v>
       </x:c>
       <x:c r="U9" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-012;fusion-src-014;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-012;fusion-src-014</x:v>
       </x:c>
       <x:c r="V9" s="31" t="str">
         <x:v>observed component/facility milestones with scope limits</x:v>
@@ -13495,7 +14329,7 @@
         <x:v>The verified source set directly informs physical flexibility or elapsed-time floors for Magnets within the frozen research-to-pilot pathway.</x:v>
       </x:c>
       <x:c r="AA9" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-012;fusion-src-014;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-012;fusion-src-014</x:v>
       </x:c>
       <x:c r="AB9" s="31" t="str">
         <x:v>observed component/facility milestones with scope limits</x:v>
@@ -13513,7 +14347,7 @@
         <x:v>The verified source set complicates any simple claim about intrinsic error tolerance for Magnets; physical scope and lifecycle distinctions remain load-bearing.</x:v>
       </x:c>
       <x:c r="AG9" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-012;fusion-src-014;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-012;fusion-src-014</x:v>
       </x:c>
       <x:c r="AH9" s="31" t="str">
         <x:v>observed component/facility milestones with scope limits</x:v>
@@ -13991,7 +14825,7 @@
         <x:v>The verified source set complicates any simple claim about information intensity for Component fabrication; physical scope and lifecycle distinctions remain load-bearing.</x:v>
       </x:c>
       <x:c r="I14" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-014;fusion-src-016;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-014;fusion-src-016</x:v>
       </x:c>
       <x:c r="J14" s="31" t="str">
         <x:v>observed fusion-component manufacture and acceptance milestones</x:v>
@@ -14009,7 +14843,7 @@
         <x:v>The verified source set directly informs feedback speed for Component fabrication within the frozen research-to-pilot pathway.</x:v>
       </x:c>
       <x:c r="O14" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-014;fusion-src-016;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-014;fusion-src-016</x:v>
       </x:c>
       <x:c r="P14" s="31" t="str">
         <x:v>observed fusion-component manufacture and acceptance milestones</x:v>
@@ -14027,7 +14861,7 @@
         <x:v>The verified source set complicates any simple claim about experiment affordability and throughput for Component fabrication; physical scope and lifecycle distinctions remain load-bearing.</x:v>
       </x:c>
       <x:c r="U14" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-014;fusion-src-016;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-014;fusion-src-016</x:v>
       </x:c>
       <x:c r="V14" s="31" t="str">
         <x:v>observed fusion-component manufacture and acceptance milestones</x:v>
@@ -14045,7 +14879,7 @@
         <x:v>The verified source set directly informs physical flexibility or elapsed-time floors for Component fabrication within the frozen research-to-pilot pathway.</x:v>
       </x:c>
       <x:c r="AA14" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-014;fusion-src-016;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-014;fusion-src-016</x:v>
       </x:c>
       <x:c r="AB14" s="31" t="str">
         <x:v>observed fusion-component manufacture and acceptance milestones</x:v>
@@ -14063,7 +14897,7 @@
         <x:v>The verified source set directly informs intrinsic error tolerance for Component fabrication within the frozen research-to-pilot pathway.</x:v>
       </x:c>
       <x:c r="AG14" s="31" t="str">
-        <x:v>fusion-src-002;fusion-src-014;fusion-src-016;fusion-src-030</x:v>
+        <x:v>fusion-src-002;fusion-src-014;fusion-src-016</x:v>
       </x:c>
       <x:c r="AH14" s="31" t="str">
         <x:v>observed fusion-component manufacture and acceptance milestones</x:v>
@@ -14101,7 +14935,7 @@
         <x:v>The verified source set complicates any simple claim about information intensity for Construction; physical scope and lifecycle distinctions remain load-bearing.</x:v>
       </x:c>
       <x:c r="I15" s="31" t="str">
-        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-033;fusion-src-036</x:v>
+        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-030;fusion-src-033;fusion-src-036;fusion-src-037</x:v>
       </x:c>
       <x:c r="J15" s="31" t="str">
         <x:v>observed facility milestones plus official baseline</x:v>
@@ -14119,7 +14953,7 @@
         <x:v>The verified source set directly informs feedback speed for Construction within the frozen research-to-pilot pathway.</x:v>
       </x:c>
       <x:c r="O15" s="31" t="str">
-        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-033;fusion-src-036</x:v>
+        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-030;fusion-src-033;fusion-src-036;fusion-src-037</x:v>
       </x:c>
       <x:c r="P15" s="31" t="str">
         <x:v>observed facility milestones plus official baseline</x:v>
@@ -14137,7 +14971,7 @@
         <x:v>The verified source set complicates any simple claim about experiment affordability and throughput for Construction; physical scope and lifecycle distinctions remain load-bearing.</x:v>
       </x:c>
       <x:c r="U15" s="31" t="str">
-        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-033;fusion-src-036</x:v>
+        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-030;fusion-src-033;fusion-src-036;fusion-src-037</x:v>
       </x:c>
       <x:c r="V15" s="31" t="str">
         <x:v>observed facility milestones plus official baseline</x:v>
@@ -14155,7 +14989,7 @@
         <x:v>The verified source set directly informs physical flexibility or elapsed-time floors for Construction within the frozen research-to-pilot pathway.</x:v>
       </x:c>
       <x:c r="AA15" s="31" t="str">
-        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-033;fusion-src-036</x:v>
+        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-030;fusion-src-033;fusion-src-036;fusion-src-037</x:v>
       </x:c>
       <x:c r="AB15" s="31" t="str">
         <x:v>observed facility milestones plus official baseline</x:v>
@@ -14173,7 +15007,7 @@
         <x:v>The verified source set directly informs intrinsic error tolerance for Construction within the frozen research-to-pilot pathway.</x:v>
       </x:c>
       <x:c r="AG15" s="31" t="str">
-        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-033;fusion-src-036</x:v>
+        <x:v>fusion-src-010;fusion-src-012;fusion-src-016;fusion-src-030;fusion-src-033;fusion-src-036;fusion-src-037</x:v>
       </x:c>
       <x:c r="AH15" s="31" t="str">
         <x:v>observed facility milestones plus official baseline</x:v>
@@ -14405,7 +15239,7 @@
         <x:v>targeted_primary_source_search_only_if_load_bearing</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="194.39999389648438" hidden="0" customHeight="1">
+    <x:row r="18" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A18" s="31" t="str">
         <x:v>sp-0030</x:v>
       </x:c>
@@ -14434,7 +15268,7 @@
         <x:v>fusion-src-004;fusion-src-039;fusion-src-040;fusion-src-041</x:v>
       </x:c>
       <x:c r="J18" s="31" t="str">
-        <x:v>enacted authority and proposed framework; no pilot-plant licence case</x:v>
+        <x:v>enacted law and proposed-rule status; no comparable pilot-plant licence-duration case</x:v>
       </x:c>
       <x:c r="K18" s="31" t="str">
         <x:v>available_evidence_does_not_resolve_scope_or_lifecycle_confounds</x:v>
@@ -14443,19 +15277,19 @@
         <x:v>preserve_complication_for_domain_review</x:v>
       </x:c>
       <x:c r="M18" s="31" t="str">
-        <x:v>directly supported</x:v>
+        <x:v>contradicted or complicated</x:v>
       </x:c>
       <x:c r="N18" s="31" t="str">
-        <x:v>The verified source set directly informs feedback speed for Licensing within the frozen research-to-pilot pathway.</x:v>
+        <x:v>The enacted-law, proposed-rule, and regulator-status sources establish legal status but do not empirically establish fusion licence-review feedback speed; the NRC rulemaking comment interval is not a plant-licence review duration.</x:v>
       </x:c>
       <x:c r="O18" s="31" t="str">
         <x:v>fusion-src-004;fusion-src-039;fusion-src-040;fusion-src-041</x:v>
       </x:c>
       <x:c r="P18" s="31" t="str">
-        <x:v>enacted authority and proposed framework; no pilot-plant licence case</x:v>
+        <x:v>enacted law and proposed-rule status; no comparable pilot-plant licence-duration case</x:v>
       </x:c>
       <x:c r="Q18" s="31" t="str">
-        <x:v>not_missing</x:v>
+        <x:v>available_evidence_does_not_resolve_scope_or_lifecycle_confounds</x:v>
       </x:c>
       <x:c r="R18" s="31" t="str">
         <x:v>regulatory_domain_review_exception</x:v>
@@ -14464,13 +15298,13 @@
         <x:v>no suitable source located</x:v>
       </x:c>
       <x:c r="T18" s="31" t="str">
-        <x:v>A bounded first-pass search located no suitable source directly supporting a claim about experiment affordability and throughput for Licensing; this is not evidence of absence.</x:v>
+        <x:v>No suitable source in this bounded pass directly establishes the affordability or throughput of a comparable fusion pilot-plant licensing review; this is not evidence of absence.</x:v>
       </x:c>
       <x:c r="U18" s="31" t="str">
         <x:v>missing</x:v>
       </x:c>
       <x:c r="V18" s="31" t="str">
-        <x:v>enacted authority and proposed framework; no pilot-plant licence case</x:v>
+        <x:v>enacted law and proposed-rule status; no comparable pilot-plant licence-duration case</x:v>
       </x:c>
       <x:c r="W18" s="31" t="str">
         <x:v>bounded_search_no_suitable_source_located_not_evidence_of_absence</x:v>
@@ -14479,34 +15313,34 @@
         <x:v>regulatory_domain_review_exception</x:v>
       </x:c>
       <x:c r="Y18" s="31" t="str">
-        <x:v>directly supported</x:v>
+        <x:v>indirectly supported/analogy</x:v>
       </x:c>
       <x:c r="Z18" s="31" t="str">
-        <x:v>The verified source set directly informs physical flexibility or elapsed-time floors for Licensing within the frozen research-to-pilot pathway.</x:v>
+        <x:v>The legal and regulatory sources provide at most indirect, partial evidence about licensing elapsed-time floors; they do not empirically prove that licensing lacks an intrinsic process constraint.</x:v>
       </x:c>
       <x:c r="AA18" s="31" t="str">
         <x:v>fusion-src-004;fusion-src-039;fusion-src-040;fusion-src-041</x:v>
       </x:c>
       <x:c r="AB18" s="31" t="str">
-        <x:v>enacted authority and proposed framework; no pilot-plant licence case</x:v>
+        <x:v>enacted law and proposed-rule status; no comparable pilot-plant licence-duration case</x:v>
       </x:c>
       <x:c r="AC18" s="31" t="str">
-        <x:v>not_missing</x:v>
+        <x:v>only_adjacent_stage_or_pathway_evidence_located</x:v>
       </x:c>
       <x:c r="AD18" s="31" t="str">
-        <x:v>domain_review_before_any_S_adjudication</x:v>
+        <x:v>seek_stage_and_lifecycle_matched_primary_evidence</x:v>
       </x:c>
       <x:c r="AE18" s="31" t="str">
         <x:v>indirectly supported/analogy</x:v>
       </x:c>
       <x:c r="AF18" s="31" t="str">
-        <x:v>The verified source set informs intrinsic error tolerance for Licensing only by bounded analogy or adjacent-stage evidence.</x:v>
+        <x:v>The legal and regulatory sources inform licensing error tolerance only indirectly and remain domain-sensitive; no completed comparable fusion licence case resolves the issue.</x:v>
       </x:c>
       <x:c r="AG18" s="31" t="str">
         <x:v>fusion-src-004;fusion-src-039;fusion-src-040;fusion-src-041</x:v>
       </x:c>
       <x:c r="AH18" s="31" t="str">
-        <x:v>enacted authority and proposed framework; no pilot-plant licence case</x:v>
+        <x:v>enacted law and proposed-rule status; no comparable pilot-plant licence-duration case</x:v>
       </x:c>
       <x:c r="AI18" s="31" t="str">
         <x:v>only_adjacent_stage_or_pathway_evidence_located</x:v>
@@ -14628,7 +15462,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raccabc0886724d29"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re470a799bf934203"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14681,7 +15515,7 @@
         <x:v>notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="162" hidden="0" customHeight="1">
+    <x:row r="2" ht="226.8000030517578" hidden="0" customHeight="1">
       <x:c r="A2" s="31" t="str">
         <x:v>promotion-exception-001</x:v>
       </x:c>
@@ -14698,10 +15532,10 @@
         <x:v>S2</x:v>
       </x:c>
       <x:c r="F2" s="31" t="str">
-        <x:v>The verified source set complicates any simple claim about feedback speed for Materials qualification; physical scope and lifecycle distinctions remain load-bearing.</x:v>
+        <x:v>IFMIF-DONES design and programme-target sources directly establish a planned multi-year irradiation-and-post-irradiation-examination feedback chain for materials qualification; they do not report a completed dataset.</x:v>
       </x:c>
       <x:c r="G2" s="31" t="str">
-        <x:v>fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038 · verified_inventory_mapping</x:v>
+        <x:v>fusion-src-046;fusion-src-045;fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038 · verified_inventory_mapping</x:v>
       </x:c>
       <x:c r="H2" s="31" t="str">
         <x:v>Confirm whether the bounded source scope is sufficient for promotion review; do not select an S value here.</x:v>
@@ -14711,7 +15545,7 @@
         <x:v>Exception surfaced from the authoritative owner-routing inputs; uncontested sources are not listed here.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="162" hidden="0" customHeight="1">
+    <x:row r="3" ht="237.60000610351562" hidden="0" customHeight="1">
       <x:c r="A3" s="31" t="str">
         <x:v>promotion-exception-002</x:v>
       </x:c>
@@ -14728,10 +15562,10 @@
         <x:v>S4</x:v>
       </x:c>
       <x:c r="F3" s="31" t="str">
-        <x:v>The verified source set directly informs physical flexibility or elapsed-time floors for Materials qualification within the frozen research-to-pilot pathway.</x:v>
+        <x:v>IFMIF-DONES design and programme-target sources directly support a substantial physical materials-qualification time floor: roughly 2.5-3 full-power years of irradiation before the remaining examination and acceptance chain.</x:v>
       </x:c>
       <x:c r="G3" s="31" t="str">
-        <x:v>fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038 · verified_inventory_mapping</x:v>
+        <x:v>fusion-src-046;fusion-src-045;fusion-src-003;fusion-src-026;fusion-src-027;fusion-src-028;fusion-src-038 · verified_inventory_mapping</x:v>
       </x:c>
       <x:c r="H3" s="31" t="str">
         <x:v>Confirm whether the bounded source scope is sufficient for promotion review; do not select an S value here.</x:v>
@@ -14741,7 +15575,7 @@
         <x:v>Exception surfaced from the authoritative owner-routing inputs; uncontested sources are not listed here.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="129.60000610351562" hidden="0" customHeight="1">
+    <x:row r="4" ht="248.39999389648438" hidden="0" customHeight="1">
       <x:c r="A4" s="31" t="str">
         <x:v>promotion-exception-003</x:v>
       </x:c>
@@ -14758,7 +15592,7 @@
         <x:v>S2</x:v>
       </x:c>
       <x:c r="F4" s="31" t="str">
-        <x:v>The verified source set directly informs feedback speed for Licensing within the frozen research-to-pilot pathway.</x:v>
+        <x:v>The enacted-law, proposed-rule, and regulator-status sources establish legal status but do not empirically establish fusion licence-review feedback speed; the NRC rulemaking comment interval is not a plant-licence review duration.</x:v>
       </x:c>
       <x:c r="G4" s="31" t="str">
         <x:v>fusion-src-004;fusion-src-039;fusion-src-040;fusion-src-041 · verified_inventory_mapping</x:v>
@@ -14788,7 +15622,7 @@
         <x:v>S3</x:v>
       </x:c>
       <x:c r="F5" s="31" t="str">
-        <x:v>A bounded first-pass search located no suitable source directly supporting a claim about experiment affordability and throughput for Licensing; this is not evidence of absence.</x:v>
+        <x:v>No suitable source in this bounded pass directly establishes the affordability or throughput of a comparable fusion pilot-plant licensing review; this is not evidence of absence.</x:v>
       </x:c>
       <x:c r="G5" s="31" t="str">
         <x:v>missing · unresolved_bounded_search</x:v>
@@ -14801,7 +15635,7 @@
         <x:v>Exception surfaced from the authoritative owner-routing inputs; uncontested sources are not listed here.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="118.80000305175781" hidden="0" customHeight="1">
+    <x:row r="6" ht="205.1999969482422" hidden="0" customHeight="1">
       <x:c r="A6" s="31" t="str">
         <x:v>promotion-exception-005</x:v>
       </x:c>
@@ -14818,7 +15652,7 @@
         <x:v>S5</x:v>
       </x:c>
       <x:c r="F6" s="31" t="str">
-        <x:v>The verified source set informs intrinsic error tolerance for Licensing only by bounded analogy or adjacent-stage evidence.</x:v>
+        <x:v>The legal and regulatory sources inform licensing error tolerance only indirectly and remain domain-sensitive; no completed comparable fusion licence case resolves the issue.</x:v>
       </x:c>
       <x:c r="G6" s="31" t="str">
         <x:v>fusion-src-004;fusion-src-039;fusion-src-040;fusion-src-041 · verified_inventory_mapping</x:v>
@@ -14929,7 +15763,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09b2ae8e59114d18"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd07e02f135ba4e92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15076,502 +15910,379 @@
         <x:v>Do not extrapolate to plant construction or commissioning.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="129.60000610351562" hidden="0" customHeight="1">
+    <x:row r="4" ht="151.1999969482422" hidden="0" customHeight="1">
       <x:c r="A4" s="31" t="str">
-        <x:v>fusion-rej-003</x:v>
+        <x:v>fusion-rej-005</x:v>
       </x:c>
       <x:c r="B4" s="31" t="str">
-        <x:v>unassigned_pack_table</x:v>
+        <x:v>S-AI-KSTAR-D3D</x:v>
       </x:c>
       <x:c r="C4" s="31" t="str">
-        <x:v>fusion-src-023</x:v>
+        <x:v>fusion-src-019</x:v>
       </x:c>
       <x:c r="D4" s="31" t="str">
-        <x:v>HEAT-ML simulation claim</x:v>
+        <x:v>Simplified 'up to 90%' fusion-performance improvement</x:v>
       </x:c>
       <x:c r="E4" s="31" t="str">
-        <x:v>https://www.pppl.gov/news/2026</x:v>
+        <x:v>https://doi.org/10.1038/s41467-024-48415-w</x:v>
       </x:c>
       <x:c r="F4" s="31" t="str">
-        <x:v>deferred</x:v>
+        <x:v>rejected_as_worded</x:v>
       </x:c>
       <x:c r="G4" s="31" t="str">
-        <x:v>unverified_url_or_doi</x:v>
+        <x:v>denominator_and_metric_mismatch</x:v>
       </x:c>
       <x:c r="H4" s="31" t="str">
-        <x:v>The pack did not provide a stable PPPL article URL or DOI, and the exact publisher page/paper could not be recovered in the bounded pass.</x:v>
+        <x:v>The paper reports several device- and metric-specific changes; the pack's compressed percentage omits the exact metric, denominator, device, and condition.</x:v>
       </x:c>
       <x:c r="I4" s="31" t="str">
-        <x:v>Research lead only; no claim support or source-register promotion.</x:v>
+        <x:v>Cite the peer-reviewed cross-device experiment qualitatively or extract a metric-specific value with a Results/figure locator.</x:v>
       </x:c>
       <x:c r="J4" s="31" t="str">
-        <x:v>sp-0015;sp-0023</x:v>
+        <x:v>sp-0016;sp-0017;sp-0018</x:v>
       </x:c>
       <x:c r="K4" s="31" t="str">
-        <x:v>S1;S2;S3</x:v>
+        <x:v>S2;S3</x:v>
       </x:c>
       <x:c r="L4" s="31" t="str">
         <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="M4" s="31" t="str">
-        <x:v>Verify exact Fusion Engineering and Design paper before reuse.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="162" hidden="0" customHeight="1">
+        <x:v>The source remains staged; only the simplified number is rejected.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="183.60000610351562" hidden="0" customHeight="1">
       <x:c r="A5" s="31" t="str">
-        <x:v>fusion-rej-004</x:v>
+        <x:v>fusion-rej-007</x:v>
       </x:c>
       <x:c r="B5" s="31" t="str">
-        <x:v>S-ITER-2026</x:v>
+        <x:v>S-CN-CRAFT-TF</x:v>
       </x:c>
       <x:c r="C5" s="31" t="str">
-        <x:v>fusion-src-037</x:v>
+        <x:v>fusion-src-002</x:v>
       </x:c>
       <x:c r="D5" s="31" t="str">
-        <x:v>ITER July 2026 sixth-of-nine sector count</x:v>
+        <x:v>CRAFT TF system is the world's largest/strongest without a definition-matched comparison</x:v>
       </x:c>
       <x:c r="E5" s="31" t="str">
-        <x:v>https://www.iter.org/project/assembly-overview</x:v>
+        <x:v>https://www.ipp.cas.cn/hnxny/kyxm/202603/t20260309_825283.html</x:v>
       </x:c>
       <x:c r="F5" s="31" t="str">
-        <x:v>deferred</x:v>
+        <x:v>rejected_as_worded</x:v>
       </x:c>
       <x:c r="G5" s="31" t="str">
-        <x:v>unverified_numeric_claim</x:v>
+        <x:v>unsupported_superlative</x:v>
       </x:c>
       <x:c r="H5" s="31" t="str">
-        <x:v>The stable assembly page verifies phase topology but not the pack's July-2026 sixth-of-nine numerical claim; the exact original news page was not recovered.</x:v>
+        <x:v>Dimensions, mass, current, stored energy, and field are different metrics; no stable comparison table establishes a single common 'largest/strongest' category.</x:v>
       </x:c>
       <x:c r="I5" s="31" t="str">
-        <x:v>Use the stable page for assembly and commissioning phase definitions only.</x:v>
+        <x:v>Use individual parameters with their exact component definition and article locator.</x:v>
       </x:c>
       <x:c r="J5" s="31" t="str">
-        <x:v>sp-0026;sp-0027;sp-0028</x:v>
+        <x:v>sp-0021;sp-0026</x:v>
       </x:c>
       <x:c r="K5" s="31" t="str">
-        <x:v>S2;S3;S4</x:v>
+        <x:v>S3;S4</x:v>
       </x:c>
       <x:c r="L5" s="31" t="str">
         <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="M5" s="31" t="str">
-        <x:v>No numerical promotion without a precise locator.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="151.1999969482422" hidden="0" customHeight="1">
+        <x:v>The component milestone remains staged.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="183.60000610351562" hidden="0" customHeight="1">
       <x:c r="A6" s="31" t="str">
-        <x:v>fusion-rej-005</x:v>
+        <x:v>fusion-rej-008</x:v>
       </x:c>
       <x:c r="B6" s="31" t="str">
-        <x:v>S-AI-KSTAR-D3D</x:v>
+        <x:v>S-CN-MFG</x:v>
       </x:c>
       <x:c r="C6" s="31" t="str">
-        <x:v>fusion-src-019</x:v>
+        <x:v>missing</x:v>
       </x:c>
       <x:c r="D6" s="31" t="str">
-        <x:v>Simplified 'up to 90%' fusion-performance improvement</x:v>
+        <x:v>Aggregate Chinese steel, cement, reactor count, or heavy-industry scale as fusion-grade capacity</x:v>
       </x:c>
       <x:c r="E6" s="31" t="str">
-        <x:v>https://doi.org/10.1038/s41467-024-48415-w</x:v>
+        <x:v>missing</x:v>
       </x:c>
       <x:c r="F6" s="31" t="str">
-        <x:v>rejected_as_worded</x:v>
+        <x:v>rejected</x:v>
       </x:c>
       <x:c r="G6" s="31" t="str">
-        <x:v>denominator_and_metric_mismatch</x:v>
+        <x:v>generic_industrial_scale_scope_mismatch</x:v>
       </x:c>
       <x:c r="H6" s="31" t="str">
-        <x:v>The paper reports several device- and metric-specific changes; the pack's compressed percentage omits the exact metric, denominator, device, and condition.</x:v>
+        <x:v>Bulk industrial output does not establish qualified fusion magnets, RAFM/advanced alloys, nuclear welding/NDE, blankets, tritium systems, or plasma-facing components.</x:v>
       </x:c>
       <x:c r="I6" s="31" t="str">
-        <x:v>Cite the peer-reviewed cross-device experiment qualitatively or extract a metric-specific value with a Results/figure locator.</x:v>
+        <x:v>Adjacent industrial-mobilization context only, explicitly outside profile evidence.</x:v>
       </x:c>
       <x:c r="J6" s="31" t="str">
-        <x:v>sp-0016;sp-0017;sp-0018</x:v>
+        <x:v>sp-0020;sp-0021;sp-0023;sp-0024;sp-0025;sp-0026;sp-0027</x:v>
       </x:c>
       <x:c r="K6" s="31" t="str">
-        <x:v>S2;S3</x:v>
+        <x:v>S2;S3;S4;S5</x:v>
       </x:c>
       <x:c r="L6" s="31" t="str">
         <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="M6" s="31" t="str">
-        <x:v>The source remains staged; only the simplified number is rejected.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="108" hidden="0" customHeight="1">
+        <x:v>No national score or bilateral ranking follows from adjacent scale.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="172.8000030517578" hidden="0" customHeight="1">
       <x:c r="A7" s="31" t="str">
-        <x:v>fusion-rej-006</x:v>
+        <x:v>fusion-rej-009</x:v>
       </x:c>
       <x:c r="B7" s="31" t="str">
-        <x:v>S-US-NSTXU</x:v>
+        <x:v>S-CN-HH70-XH;S-CN-HH70-CO</x:v>
       </x:c>
       <x:c r="C7" s="31" t="str">
-        <x:v>fusion-src-030</x:v>
+        <x:v>fusion-src-011;fusion-src-012</x:v>
       </x:c>
       <x:c r="D7" s="31" t="str">
-        <x:v>NSTX-U is 93% complete</x:v>
+        <x:v>HH70's roughly two-year build as a fusion power-plant construction floor</x:v>
       </x:c>
       <x:c r="E7" s="31" t="str">
-        <x:v>https://www.pppl.gov/news/2026/delivery-magnet-bundle-signals-new-age-fusion-research</x:v>
+        <x:v>https://www.sh.news.cn/20260410/696d097c4a6c41b9af5f654314252a04/c.html</x:v>
       </x:c>
       <x:c r="F7" s="31" t="str">
-        <x:v>deferred</x:v>
+        <x:v>rejected</x:v>
       </x:c>
       <x:c r="G7" s="31" t="str">
-        <x:v>unverified_numeric_claim</x:v>
+        <x:v>lifecycle_and_system_scope_mismatch</x:v>
       </x:c>
       <x:c r="H7" s="31" t="str">
-        <x:v>The verified PPPL page supports a central-magnet delivery and a 2027 experiment target, but not the 93% value.</x:v>
+        <x:v>HH70 is a small, non-DT research tokamak without a breeder blanket, turbine, integrated tritium plant, or commercial nuclear commissioning.</x:v>
       </x:c>
       <x:c r="I7" s="31" t="str">
-        <x:v>Use the verified delivery milestone and target with their exact status labels.</x:v>
+        <x:v>Optimistic analogue for small research-device iteration only.</x:v>
       </x:c>
       <x:c r="J7" s="31" t="str">
-        <x:v>sp-0021;sp-0026;sp-0027;sp-0028</x:v>
+        <x:v>sp-0027;sp-0028</x:v>
       </x:c>
       <x:c r="K7" s="31" t="str">
-        <x:v>S2;S3;S4</x:v>
+        <x:v>S2;S4</x:v>
       </x:c>
       <x:c r="L7" s="31" t="str">
         <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="M7" s="31" t="str">
-        <x:v>Do not infer overall completion percentage.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="183.60000610351562" hidden="0" customHeight="1">
+        <x:v>Do not transfer elapsed time to a pilot plant.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="162" hidden="0" customHeight="1">
       <x:c r="A8" s="31" t="str">
-        <x:v>fusion-rej-007</x:v>
+        <x:v>fusion-rej-010</x:v>
       </x:c>
       <x:c r="B8" s="31" t="str">
-        <x:v>S-CN-CRAFT-TF</x:v>
+        <x:v>S-CN-EAST;S-CN-HH70-XH;S-DE-W7X</x:v>
       </x:c>
       <x:c r="C8" s="31" t="str">
-        <x:v>fusion-src-002</x:v>
+        <x:v>fusion-src-001;fusion-src-011;fusion-src-032</x:v>
       </x:c>
       <x:c r="D8" s="31" t="str">
-        <x:v>CRAFT TF system is the world's largest/strongest without a definition-matched comparison</x:v>
+        <x:v>Long plasma duration as commercial reliability or availability</x:v>
       </x:c>
       <x:c r="E8" s="31" t="str">
-        <x:v>https://www.ipp.cas.cn/hnxny/kyxm/202603/t20260309_825283.html</x:v>
+        <x:v>https://www.ipp.cas.cn/xwdt/ttxw/202501/t20250120_410191.html</x:v>
       </x:c>
       <x:c r="F8" s="31" t="str">
-        <x:v>rejected_as_worded</x:v>
+        <x:v>rejected</x:v>
       </x:c>
       <x:c r="G8" s="31" t="str">
-        <x:v>unsupported_superlative</x:v>
+        <x:v>metric_category_error</x:v>
       </x:c>
       <x:c r="H8" s="31" t="str">
-        <x:v>Dimensions, mass, current, stored energy, and field are different metrics; no stable comparison table establishes a single common 'largest/strongest' category.</x:v>
+        <x:v>Pulse duration and energy-turnover metrics omit blanket life, tritium-plant availability, component replacement, turbine/grid systems, downtime, and capacity factor.</x:v>
       </x:c>
       <x:c r="I8" s="31" t="str">
-        <x:v>Use individual parameters with their exact component definition and article locator.</x:v>
+        <x:v>Plasma/facility milestone with device, discharge, and metric definitions preserved.</x:v>
       </x:c>
       <x:c r="J8" s="31" t="str">
-        <x:v>sp-0021;sp-0026</x:v>
+        <x:v>sp-0029</x:v>
       </x:c>
       <x:c r="K8" s="31" t="str">
-        <x:v>S3;S4</x:v>
+        <x:v>S2;S3;S4;S5</x:v>
       </x:c>
       <x:c r="L8" s="31" t="str">
         <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="M8" s="31" t="str">
-        <x:v>The component milestone remains staged.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="183.60000610351562" hidden="0" customHeight="1">
+        <x:v>No evidence of plant availability is implied.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="172.8000030517578" hidden="0" customHeight="1">
       <x:c r="A9" s="31" t="str">
-        <x:v>fusion-rej-008</x:v>
+        <x:v>fusion-rej-011</x:v>
       </x:c>
       <x:c r="B9" s="31" t="str">
-        <x:v>S-CN-MFG</x:v>
+        <x:v>S-US-MPEX</x:v>
       </x:c>
       <x:c r="C9" s="31" t="str">
-        <x:v>missing</x:v>
+        <x:v>fusion-src-026</x:v>
       </x:c>
       <x:c r="D9" s="31" t="str">
-        <x:v>Aggregate Chinese steel, cement, reactor count, or heavy-industry scale as fusion-grade capacity</x:v>
+        <x:v>MPEX as an operating fusion-spectrum neutron qualification facility</x:v>
       </x:c>
       <x:c r="E9" s="31" t="str">
-        <x:v>missing</x:v>
+        <x:v>https://mpex.ornl.gov/murf-2026/</x:v>
       </x:c>
       <x:c r="F9" s="31" t="str">
-        <x:v>rejected</x:v>
+        <x:v>rejected_as_worded</x:v>
       </x:c>
       <x:c r="G9" s="31" t="str">
-        <x:v>generic_industrial_scale_scope_mismatch</x:v>
+        <x:v>facility_function_scope_mismatch</x:v>
       </x:c>
       <x:c r="H9" s="31" t="str">
-        <x:v>Bulk industrial output does not establish qualified fusion magnets, RAFM/advanced alloys, nuclear welding/NDE, blankets, tritium systems, or plasma-facing components.</x:v>
+        <x:v>MPEX is a plasma-materials exposure facility under assembly; it can test already neutron-irradiated specimens but is not itself a fusion-spectrum neutron source.</x:v>
       </x:c>
       <x:c r="I9" s="31" t="str">
-        <x:v>Adjacent industrial-mobilization context only, explicitly outside profile evidence.</x:v>
+        <x:v>Official intended capability for reactor-edge plasma exposure.</x:v>
       </x:c>
       <x:c r="J9" s="31" t="str">
-        <x:v>sp-0020;sp-0021;sp-0023;sp-0024;sp-0025;sp-0026;sp-0027</x:v>
+        <x:v>sp-0020;sp-0023</x:v>
       </x:c>
       <x:c r="K9" s="31" t="str">
-        <x:v>S2;S3;S4;S5</x:v>
+        <x:v>S2;S3;S4</x:v>
       </x:c>
       <x:c r="L9" s="31" t="str">
         <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="M9" s="31" t="str">
-        <x:v>No national score or bilateral ranking follows from adjacent scale.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="172.8000030517578" hidden="0" customHeight="1">
+        <x:v>Do not call intended capability completed qualification.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="129.60000610351562" hidden="0" customHeight="1">
       <x:c r="A10" s="31" t="str">
-        <x:v>fusion-rej-009</x:v>
+        <x:v>fusion-rej-012</x:v>
       </x:c>
       <x:c r="B10" s="31" t="str">
-        <x:v>S-CN-HH70-XH;S-CN-HH70-CO</x:v>
+        <x:v>S-IAEA-SAFE</x:v>
       </x:c>
       <x:c r="C10" s="31" t="str">
-        <x:v>fusion-src-011;fusion-src-012</x:v>
+        <x:v>fusion-src-041</x:v>
       </x:c>
       <x:c r="D10" s="31" t="str">
-        <x:v>HH70's roughly two-year build as a fusion power-plant construction floor</x:v>
+        <x:v>A completed fusion-specific IAEA safety standard exists</x:v>
       </x:c>
       <x:c r="E10" s="31" t="str">
-        <x:v>https://www.sh.news.cn/20260410/696d097c4a6c41b9af5f654314252a04/c.html</x:v>
+        <x:v>https://www.iaea.org/sites/default/files/25/02/evt2405228_information_sheet_.pdf</x:v>
       </x:c>
       <x:c r="F10" s="31" t="str">
-        <x:v>rejected</x:v>
+        <x:v>rejected_as_worded</x:v>
       </x:c>
       <x:c r="G10" s="31" t="str">
-        <x:v>lifecycle_and_system_scope_mismatch</x:v>
+        <x:v>programme_announcement_not_standard</x:v>
       </x:c>
       <x:c r="H10" s="31" t="str">
-        <x:v>HH70 is a small, non-DT research tokamak without a breeder blanket, turbine, integrated tritium plant, or commercial nuclear commissioning.</x:v>
+        <x:v>The verified document describes a meeting and a safety report in development; it is not a published fusion-specific Safety Standard.</x:v>
       </x:c>
       <x:c r="I10" s="31" t="str">
-        <x:v>Optimistic analogue for small research-device iteration only.</x:v>
+        <x:v>Evidence of international safety/regulatory work in progress.</x:v>
       </x:c>
       <x:c r="J10" s="31" t="str">
-        <x:v>sp-0027;sp-0028</x:v>
+        <x:v>sp-0030</x:v>
       </x:c>
       <x:c r="K10" s="31" t="str">
-        <x:v>S2;S4</x:v>
+        <x:v>S2;S3;S4;S5</x:v>
       </x:c>
       <x:c r="L10" s="31" t="str">
         <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="M10" s="31" t="str">
-        <x:v>Do not transfer elapsed time to a pilot plant.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="162" hidden="0" customHeight="1">
+        <x:v>Keep IAEA general safety standards separate from fusion-specific guidance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="140.39999389648438" hidden="0" customHeight="1">
       <x:c r="A11" s="31" t="str">
-        <x:v>fusion-rej-010</x:v>
+        <x:v>fusion-rej-013</x:v>
       </x:c>
       <x:c r="B11" s="31" t="str">
-        <x:v>S-CN-EAST;S-CN-HH70-XH;S-DE-W7X</x:v>
+        <x:v>S-US-SPARC;S-UK-STEP;S-TYPEONE;S-PROXIMA</x:v>
       </x:c>
       <x:c r="C11" s="31" t="str">
-        <x:v>fusion-src-001;fusion-src-011;fusion-src-032</x:v>
+        <x:v>fusion-src-031;fusion-src-035;fusion-src-043;fusion-src-044</x:v>
       </x:c>
       <x:c r="D11" s="31" t="str">
-        <x:v>Long plasma duration as commercial reliability or availability</x:v>
+        <x:v>Company or official programme dates as observed fusion-grid outcomes</x:v>
       </x:c>
       <x:c r="E11" s="31" t="str">
-        <x:v>https://www.ipp.cas.cn/xwdt/ttxw/202501/t20250120_410191.html</x:v>
+        <x:v>multiple_verified_primary_pages</x:v>
       </x:c>
       <x:c r="F11" s="31" t="str">
         <x:v>rejected</x:v>
       </x:c>
       <x:c r="G11" s="31" t="str">
-        <x:v>metric_category_error</x:v>
+        <x:v>target_not_observed_outcome</x:v>
       </x:c>
       <x:c r="H11" s="31" t="str">
-        <x:v>Pulse duration and energy-turnover metrics omit blanket life, tritium-plant availability, component replacement, turbine/grid systems, downtime, and capacity factor.</x:v>
+        <x:v>Targets and programme announcements do not demonstrate net energy, electricity export, fuel self-sufficiency, availability, or grid connection.</x:v>
       </x:c>
       <x:c r="I11" s="31" t="str">
-        <x:v>Plasma/facility milestone with device, discharge, and metric definitions preserved.</x:v>
+        <x:v>Target tracking with owner, date, pathway, and target status preserved.</x:v>
       </x:c>
       <x:c r="J11" s="31" t="str">
-        <x:v>sp-0029</x:v>
+        <x:v>sp-0027;sp-0028;sp-0031</x:v>
       </x:c>
       <x:c r="K11" s="31" t="str">
-        <x:v>S2;S3;S4;S5</x:v>
+        <x:v>S2;S3;S4</x:v>
       </x:c>
       <x:c r="L11" s="31" t="str">
         <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="M11" s="31" t="str">
-        <x:v>No evidence of plant availability is implied.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="172.8000030517578" hidden="0" customHeight="1">
+        <x:v>No target is typed as an observed result.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="140.39999389648438" hidden="0" customHeight="1">
       <x:c r="A12" s="31" t="str">
-        <x:v>fusion-rej-011</x:v>
+        <x:v>fusion-rej-014</x:v>
       </x:c>
       <x:c r="B12" s="31" t="str">
-        <x:v>S-US-MPEX</x:v>
+        <x:v>all</x:v>
       </x:c>
       <x:c r="C12" s="31" t="str">
-        <x:v>fusion-src-026</x:v>
+        <x:v>missing</x:v>
       </x:c>
       <x:c r="D12" s="31" t="str">
-        <x:v>MPEX as an operating fusion-spectrum neutron qualification facility</x:v>
+        <x:v>No evidence located as evidence of absence</x:v>
       </x:c>
       <x:c r="E12" s="31" t="str">
-        <x:v>https://mpex.ornl.gov/murf-2026/</x:v>
+        <x:v>missing</x:v>
       </x:c>
       <x:c r="F12" s="31" t="str">
-        <x:v>rejected_as_worded</x:v>
+        <x:v>rejected</x:v>
       </x:c>
       <x:c r="G12" s="31" t="str">
-        <x:v>facility_function_scope_mismatch</x:v>
+        <x:v>absence_inference_not_supported</x:v>
       </x:c>
       <x:c r="H12" s="31" t="str">
-        <x:v>MPEX is a plasma-materials exposure facility under assembly; it can test already neutron-irradiated specimens but is not itself a fusion-spectrum neutron source.</x:v>
+        <x:v>A bounded search result does not establish that evidence or capability does not exist.</x:v>
       </x:c>
       <x:c r="I12" s="31" t="str">
-        <x:v>Official intended capability for reactor-edge plasma exposure.</x:v>
+        <x:v>Report 'no suitable source located in this bounded pass' with next search action.</x:v>
       </x:c>
       <x:c r="J12" s="31" t="str">
-        <x:v>sp-0020;sp-0023</x:v>
+        <x:v>sp-0014;sp-0015;sp-0016;sp-0017;sp-0018;sp-0019;sp-0020;sp-0021;sp-0022;sp-0023;sp-0024;sp-0025;sp-0026;sp-0027;sp-0028;sp-0029;sp-0030;sp-0031</x:v>
       </x:c>
       <x:c r="K12" s="31" t="str">
-        <x:v>S2;S3;S4</x:v>
+        <x:v>S1;S2;S3;S4;S5</x:v>
       </x:c>
       <x:c r="L12" s="31" t="str">
         <x:v>2026-08-31</x:v>
       </x:c>
       <x:c r="M12" s="31" t="str">
-        <x:v>Do not call intended capability completed qualification.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="129.60000610351562" hidden="0" customHeight="1">
-      <x:c r="A13" s="31" t="str">
-        <x:v>fusion-rej-012</x:v>
-      </x:c>
-      <x:c r="B13" s="31" t="str">
-        <x:v>S-IAEA-SAFE</x:v>
-      </x:c>
-      <x:c r="C13" s="31" t="str">
-        <x:v>fusion-src-041</x:v>
-      </x:c>
-      <x:c r="D13" s="31" t="str">
-        <x:v>A completed fusion-specific IAEA safety standard exists</x:v>
-      </x:c>
-      <x:c r="E13" s="31" t="str">
-        <x:v>https://www.iaea.org/sites/default/files/25/02/evt2405228_information_sheet_.pdf</x:v>
-      </x:c>
-      <x:c r="F13" s="31" t="str">
-        <x:v>rejected_as_worded</x:v>
-      </x:c>
-      <x:c r="G13" s="31" t="str">
-        <x:v>programme_announcement_not_standard</x:v>
-      </x:c>
-      <x:c r="H13" s="31" t="str">
-        <x:v>The verified document describes a meeting and a safety report in development; it is not a published fusion-specific Safety Standard.</x:v>
-      </x:c>
-      <x:c r="I13" s="31" t="str">
-        <x:v>Evidence of international safety/regulatory work in progress.</x:v>
-      </x:c>
-      <x:c r="J13" s="31" t="str">
-        <x:v>sp-0030</x:v>
-      </x:c>
-      <x:c r="K13" s="31" t="str">
-        <x:v>S2;S3;S4;S5</x:v>
-      </x:c>
-      <x:c r="L13" s="31" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="M13" s="31" t="str">
-        <x:v>Keep IAEA general safety standards separate from fusion-specific guidance.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="140.39999389648438" hidden="0" customHeight="1">
-      <x:c r="A14" s="31" t="str">
-        <x:v>fusion-rej-013</x:v>
-      </x:c>
-      <x:c r="B14" s="31" t="str">
-        <x:v>S-US-SPARC;S-UK-STEP;S-TYPEONE;S-PROXIMA</x:v>
-      </x:c>
-      <x:c r="C14" s="31" t="str">
-        <x:v>fusion-src-031;fusion-src-035;fusion-src-043;fusion-src-044</x:v>
-      </x:c>
-      <x:c r="D14" s="31" t="str">
-        <x:v>Company or official programme dates as observed fusion-grid outcomes</x:v>
-      </x:c>
-      <x:c r="E14" s="31" t="str">
-        <x:v>multiple_verified_primary_pages</x:v>
-      </x:c>
-      <x:c r="F14" s="31" t="str">
-        <x:v>rejected</x:v>
-      </x:c>
-      <x:c r="G14" s="31" t="str">
-        <x:v>target_not_observed_outcome</x:v>
-      </x:c>
-      <x:c r="H14" s="31" t="str">
-        <x:v>Targets and programme announcements do not demonstrate net energy, electricity export, fuel self-sufficiency, availability, or grid connection.</x:v>
-      </x:c>
-      <x:c r="I14" s="31" t="str">
-        <x:v>Target tracking with owner, date, pathway, and target status preserved.</x:v>
-      </x:c>
-      <x:c r="J14" s="31" t="str">
-        <x:v>sp-0027;sp-0028;sp-0031</x:v>
-      </x:c>
-      <x:c r="K14" s="31" t="str">
-        <x:v>S2;S3;S4</x:v>
-      </x:c>
-      <x:c r="L14" s="31" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="M14" s="31" t="str">
-        <x:v>No target is typed as an observed result.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="140.39999389648438" hidden="0" customHeight="1">
-      <x:c r="A15" s="31" t="str">
-        <x:v>fusion-rej-014</x:v>
-      </x:c>
-      <x:c r="B15" s="31" t="str">
-        <x:v>all</x:v>
-      </x:c>
-      <x:c r="C15" s="31" t="str">
-        <x:v>missing</x:v>
-      </x:c>
-      <x:c r="D15" s="31" t="str">
-        <x:v>No evidence located as evidence of absence</x:v>
-      </x:c>
-      <x:c r="E15" s="31" t="str">
-        <x:v>missing</x:v>
-      </x:c>
-      <x:c r="F15" s="31" t="str">
-        <x:v>rejected</x:v>
-      </x:c>
-      <x:c r="G15" s="31" t="str">
-        <x:v>absence_inference_not_supported</x:v>
-      </x:c>
-      <x:c r="H15" s="31" t="str">
-        <x:v>A bounded search result does not establish that evidence or capability does not exist.</x:v>
-      </x:c>
-      <x:c r="I15" s="31" t="str">
-        <x:v>Report 'no suitable source located in this bounded pass' with next search action.</x:v>
-      </x:c>
-      <x:c r="J15" s="31" t="str">
-        <x:v>sp-0014;sp-0015;sp-0016;sp-0017;sp-0018;sp-0019;sp-0020;sp-0021;sp-0022;sp-0023;sp-0024;sp-0025;sp-0026;sp-0027;sp-0028;sp-0029;sp-0030;sp-0031</x:v>
-      </x:c>
-      <x:c r="K15" s="31" t="str">
-        <x:v>S1;S2;S3;S4;S5</x:v>
-      </x:c>
-      <x:c r="L15" s="31" t="str">
-        <x:v>2026-08-31</x:v>
-      </x:c>
-      <x:c r="M15" s="31" t="str">
         <x:v>This is a method guardrail, not a source rejection.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd7c3543b5914213"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8782310c21ae482a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15746,10 +16457,276 @@
         <x:v>Do not infer licensing throughput from rulemaking status.</x:v>
       </x:c>
     </x:row>
+    <x:row r="5" ht="216" hidden="0" customHeight="1">
+      <x:c r="A5" s="31" t="str">
+        <x:v>fusion-change-004</x:v>
+      </x:c>
+      <x:c r="B5" s="31" t="str">
+        <x:v>PRC Atomic Energy Law final-law locator</x:v>
+      </x:c>
+      <x:c r="C5" s="31" t="str">
+        <x:v>The evidence bank incorrectly cited Article 37 as the final law's fusion-specific regulatory provision.</x:v>
+      </x:c>
+      <x:c r="D5" s="31" t="str">
+        <x:v>The final law supports controlled-fusion R&amp;D in Article 14 and establishes fusion-specific supervision plus graded/classified management in Article 39; Article 37 concerns disused radioactive sources.</x:v>
+      </x:c>
+      <x:c r="E5" s="31" t="str">
+        <x:v>2025-09-12</x:v>
+      </x:c>
+      <x:c r="F5" s="31" t="str">
+        <x:v>sp-0030</x:v>
+      </x:c>
+      <x:c r="G5" s="31" t="str">
+        <x:v>S2;S3;S4;S5</x:v>
+      </x:c>
+      <x:c r="H5" s="31" t="str">
+        <x:v>p1_final_law_locator_correction</x:v>
+      </x:c>
+      <x:c r="I5" s="31" t="str">
+        <x:v>Replace the mirror and draft-number carryover with the CAEA final text and Articles 14/39.</x:v>
+      </x:c>
+      <x:c r="J5" s="31" t="str">
+        <x:v>fusion-src-004</x:v>
+      </x:c>
+      <x:c r="K5" s="31" t="str">
+        <x:v>CAEA full text, Articles 14, 37, 39, and 62.</x:v>
+      </x:c>
+      <x:c r="L5" s="31" t="str">
+        <x:v>Earlier draft numbering differed; never cite draft numbering as the final-law locator.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="183.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A6" s="31" t="str">
+        <x:v>fusion-change-005</x:v>
+      </x:c>
+      <x:c r="B6" s="31" t="str">
+        <x:v>HEAT-ML source and numeric locator</x:v>
+      </x:c>
+      <x:c r="C6" s="31" t="str">
+        <x:v>The PPPL locator and linked paper were unresolved, so the claim was deferred.</x:v>
+      </x:c>
+      <x:c r="D6" s="31" t="str">
+        <x:v>The exact PPPL page and linked Fusion Engineering and Design DOI verify the scoped 30-minute-to-milliseconds calculation result and approximately 1,000-simulation training set.</x:v>
+      </x:c>
+      <x:c r="E6" s="31" t="str">
+        <x:v>2025-08-13</x:v>
+      </x:c>
+      <x:c r="F6" s="31" t="str">
+        <x:v>sp-0015</x:v>
+      </x:c>
+      <x:c r="G6" s="31" t="str">
+        <x:v>S1;S2;S3</x:v>
+      </x:c>
+      <x:c r="H6" s="31" t="str">
+        <x:v>p1_locator_and_numeric_resolution</x:v>
+      </x:c>
+      <x:c r="I6" s="31" t="str">
+        <x:v>Stage fusion-src-023 as a simulation/design proof of concept with geometry limits.</x:v>
+      </x:c>
+      <x:c r="J6" s="31" t="str">
+        <x:v>fusion-src-023</x:v>
+      </x:c>
+      <x:c r="K6" s="31" t="str">
+        <x:v>PPPL paragraphs 95-103; DOI 10.1016/j.fusengdes.2025.115010.</x:v>
+      </x:c>
+      <x:c r="L6" s="31" t="str">
+        <x:v>Do not transfer the calculation result to plant schedule, qualification, or generic PFC performance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="129.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A7" s="31" t="str">
+        <x:v>fusion-change-006</x:v>
+      </x:c>
+      <x:c r="B7" s="31" t="str">
+        <x:v>ITER sixth sector-module milestone locator</x:v>
+      </x:c>
+      <x:c r="C7" s="31" t="str">
+        <x:v>The sixth-of-nine July 2026 count lacked a precise original locator and was deferred.</x:v>
+      </x:c>
+      <x:c r="D7" s="31" t="str">
+        <x:v>ITER's official article records the 27-28 July lift, the sixth of nine modules, and two-thirds of the plasma chamber in place.</x:v>
+      </x:c>
+      <x:c r="E7" s="31" t="str">
+        <x:v>2026-07-29</x:v>
+      </x:c>
+      <x:c r="F7" s="31" t="str">
+        <x:v>sp-0027</x:v>
+      </x:c>
+      <x:c r="G7" s="31" t="str">
+        <x:v>S2;S3;S4</x:v>
+      </x:c>
+      <x:c r="H7" s="31" t="str">
+        <x:v>p1_locator_and_numeric_resolution</x:v>
+      </x:c>
+      <x:c r="I7" s="31" t="str">
+        <x:v>Stage fusion-src-037 as an observed construction/facility milestone only.</x:v>
+      </x:c>
+      <x:c r="J7" s="31" t="str">
+        <x:v>fusion-src-037</x:v>
+      </x:c>
+      <x:c r="K7" s="31" t="str">
+        <x:v>ITER article paragraphs 162-167 and road-to-ITER milestone page.</x:v>
+      </x:c>
+      <x:c r="L7" s="31" t="str">
+        <x:v>Not an AI result, commissioning, chamber completion, or plant completion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="108" hidden="0" customHeight="1">
+      <x:c r="A8" s="31" t="str">
+        <x:v>fusion-change-007</x:v>
+      </x:c>
+      <x:c r="B8" s="31" t="str">
+        <x:v>NSTX-U 93% living-page status locator</x:v>
+      </x:c>
+      <x:c r="C8" s="31" t="str">
+        <x:v>The 93% value was not found on the previously used PPPL news article and was deferred.</x:v>
+      </x:c>
+      <x:c r="D8" s="31" t="str">
+        <x:v>PPPL's NSTX-U project page states that the Recovery Project is 93% complete as checked 2026-08-31.</x:v>
+      </x:c>
+      <x:c r="E8" s="31" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="F8" s="31" t="str">
+        <x:v>sp-0027;sp-0028</x:v>
+      </x:c>
+      <x:c r="G8" s="31" t="str">
+        <x:v>S2;S3;S4</x:v>
+      </x:c>
+      <x:c r="H8" s="31" t="str">
+        <x:v>p1_locator_and_numeric_resolution</x:v>
+      </x:c>
+      <x:c r="I8" s="31" t="str">
+        <x:v>Retain the percentage only as mutable project status with a revisit trigger.</x:v>
+      </x:c>
+      <x:c r="J8" s="31" t="str">
+        <x:v>fusion-src-030</x:v>
+      </x:c>
+      <x:c r="K8" s="31" t="str">
+        <x:v>PPPL NSTX-U page, section 'Recovery Project'.</x:v>
+      </x:c>
+      <x:c r="L8" s="31" t="str">
+        <x:v>Not completed recommissioning, a fixed historical statistic, or an experimental outcome.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="194.39999389648438" hidden="0" customHeight="1">
+      <x:c r="A9" s="31" t="str">
+        <x:v>fusion-change-008</x:v>
+      </x:c>
+      <x:c r="B9" s="31" t="str">
+        <x:v>IFMIF-DONES materials-qualification evidence</x:v>
+      </x:c>
+      <x:c r="C9" s="31" t="str">
+        <x:v>The bank lacked a targeted fusion-like neutron-source design for the materials-qualification time floor.</x:v>
+      </x:c>
+      <x:c r="D9" s="31" t="str">
+        <x:v>Peer-reviewed and official programme sources define accelerator-driven fusion-like irradiation, multi-year HFTM targets, material-specific matching, and downstream PIE.</x:v>
+      </x:c>
+      <x:c r="E9" s="31" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="F9" s="31" t="str">
+        <x:v>sp-0020</x:v>
+      </x:c>
+      <x:c r="G9" s="31" t="str">
+        <x:v>S2;S3;S4</x:v>
+      </x:c>
+      <x:c r="H9" s="31" t="str">
+        <x:v>p1_targeted_load_bearing_source_addition</x:v>
+      </x:c>
+      <x:c r="I9" s="31" t="str">
+        <x:v>Add fusion-src-045 and fusion-src-046 with under-development and no-completed-dataset limits.</x:v>
+      </x:c>
+      <x:c r="J9" s="31" t="str">
+        <x:v>fusion-src-045;fusion-src-046</x:v>
+      </x:c>
+      <x:c r="K9" s="31" t="str">
+        <x:v>DOI 10.1088/1741-4326/add172; IAEA contribution Description paragraphs 1-2.</x:v>
+      </x:c>
+      <x:c r="L9" s="31" t="str">
+        <x:v>This improves source coverage without selecting or recoding any S value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="183.60000610351562" hidden="0" customHeight="1">
+      <x:c r="A10" s="31" t="str">
+        <x:v>fusion-change-009</x:v>
+      </x:c>
+      <x:c r="B10" s="31" t="str">
+        <x:v>Licensing S2/S4 evidence overclaim</x:v>
+      </x:c>
+      <x:c r="C10" s="31" t="str">
+        <x:v>Coverage rows treated the legal/rulemaking set as direct support for licensing S2 and S4.</x:v>
+      </x:c>
+      <x:c r="D10" s="31" t="str">
+        <x:v>S2 is complicated/unresolved empirically and S4 is only indirect/partial; the 90-day comment period remains explicitly non-comparable to a plant-licence review.</x:v>
+      </x:c>
+      <x:c r="E10" s="31" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="F10" s="31" t="str">
+        <x:v>sp-0030</x:v>
+      </x:c>
+      <x:c r="G10" s="31" t="str">
+        <x:v>S2;S4</x:v>
+      </x:c>
+      <x:c r="H10" s="31" t="str">
+        <x:v>p1_claim_support_correction_not_profile_recode</x:v>
+      </x:c>
+      <x:c r="I10" s="31" t="str">
+        <x:v>Correct fusion-clm-082 and fusion-clm-084 plus dependent coverage wording.</x:v>
+      </x:c>
+      <x:c r="J10" s="31" t="str">
+        <x:v>fusion-src-004;fusion-src-039;fusion-src-040;fusion-src-041</x:v>
+      </x:c>
+      <x:c r="K10" s="31" t="str">
+        <x:v>Claim-source map and source limitations.</x:v>
+      </x:c>
+      <x:c r="L10" s="31" t="str">
+        <x:v>No S value or owner disposition changes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="151.1999969482422" hidden="0" customHeight="1">
+      <x:c r="A11" s="31" t="str">
+        <x:v>fusion-change-010</x:v>
+      </x:c>
+      <x:c r="B11" s="31" t="str">
+        <x:v>Legal/regulatory evidence category</x:v>
+      </x:c>
+      <x:c r="C11" s="31" t="str">
+        <x:v>The final PRC law and NRC rulemaking records were categorized as programme announcements.</x:v>
+      </x:c>
+      <x:c r="D11" s="31" t="str">
+        <x:v>The bank now uses observed legal/regulatory status while keeping enacted law, proposed rule, and current rulemaking status distinct.</x:v>
+      </x:c>
+      <x:c r="E11" s="31" t="str">
+        <x:v>2026-08-31</x:v>
+      </x:c>
+      <x:c r="F11" s="31" t="str">
+        <x:v>sp-0030</x:v>
+      </x:c>
+      <x:c r="G11" s="31" t="str">
+        <x:v>S2;S3;S4;S5</x:v>
+      </x:c>
+      <x:c r="H11" s="31" t="str">
+        <x:v>p1_research_bank_category_correction</x:v>
+      </x:c>
+      <x:c r="I11" s="31" t="str">
+        <x:v>Update only the research-bank taxonomy and validators.</x:v>
+      </x:c>
+      <x:c r="J11" s="31" t="str">
+        <x:v>fusion-src-004;fusion-src-039;fusion-src-040</x:v>
+      </x:c>
+      <x:c r="K11" s="31" t="str">
+        <x:v>Final law; Federal Register proposed rule; NRC status page.</x:v>
+      </x:c>
+      <x:c r="L11" s="31" t="str">
+        <x:v>The global public evidence-basis ontology is unchanged.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra951902b08e440a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9903219da4c04028"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15792,7 +16769,7 @@
         <x:v>Read-only summary.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="205.1999969482422" hidden="0" customHeight="1">
+    <x:row r="3" ht="237.60000610351562" hidden="0" customHeight="1">
       <x:c r="A3" s="31" t="str">
         <x:v>SOURCE_CANDIDATES</x:v>
       </x:c>
@@ -15803,7 +16780,7 @@
         <x:v>The source-level claim category established by the original source.</x:v>
       </x:c>
       <x:c r="D3" s="31" t="str">
-        <x:v>observed experimental result; observed facility milestone; official target; company target; programme announcement; proof of concept; model or scenario estimate; inference; commentary</x:v>
+        <x:v>observed experimental result; observed facility milestone; observed legal/regulatory status; official target; company target; programme announcement; proof of concept; model or scenario estimate; inference; commentary</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="86.4000015258789" hidden="0" customHeight="1">
@@ -15949,7 +16926,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08ed97651b15464d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf747df1df016482d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>